<commit_message>
Update: Pappu Hardware — 50 bags cement + transport + labour (21-Jun, ₹18,500)
All Transactions: 3 rows added (cement ₹18,000, transport ₹300, labour ₹200)
Payment Tracker: ₹18,500 paid by Self-GPay
Excel: 0 formula errors, 2732 formulas verified

Updated totals:
- Total Billed: ₹12,36,297 → ₹12,54,797 (+₹18,500)
- Total Paid: ₹14,38,297 → ₹14,56,797 (+₹18,500)
- Jun-2026: ₹4,06,705 → ₹4,25,205 (+₹18,500)
- Pappu Hardware: ₹4,51,130 → ₹4,69,630 billed; still ₹1,300 due (old bill 4)
- Cement on site: 250 → 300 bags

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -953,7 +953,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -1101,7 +1101,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1190,7 +1190,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1223,7 +1223,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -6451,7 +6451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q506"/>
+  <dimension ref="A1:Q509"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -20393,8 +20393,6 @@
         <f>IF(L504="","",IF(M504="",L504,L504*(1-M504)))</f>
         <v/>
       </c>
-      <c r="P504" t="inlineStr"/>
-      <c r="Q504" t="inlineStr"/>
     </row>
     <row r="505" ht="15.75" customHeight="1" s="99">
       <c r="A505" t="n">
@@ -20455,37 +20453,245 @@
         <f>IF(L505="","",IF(M505="",L505,L505*(1-M505)))</f>
         <v/>
       </c>
-      <c r="P505" t="inlineStr"/>
-      <c r="Q505" t="inlineStr"/>
     </row>
     <row r="506">
-      <c r="A506" s="60" t="inlineStr">
+      <c r="A506" t="n">
+        <v>503</v>
+      </c>
+      <c r="B506" s="127" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C506">
+        <f>IF(B506="","",TEXT(B506,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>Ultratech Super Cement 50 bags @ ₹360</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I506" t="n">
+        <v>50</v>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K506" t="n">
+        <v>360</v>
+      </c>
+      <c r="L506">
+        <f>IF(OR(I506="",K506=""),"",I506*K506)</f>
+        <v/>
+      </c>
+      <c r="N506">
+        <f>M506*L506</f>
+        <v/>
+      </c>
+      <c r="O506">
+        <f>IF(L506="","",IF(M506="",L506,L506*(1-M506)))</f>
+        <v/>
+      </c>
+      <c r="P506" t="inlineStr">
+        <is>
+          <t>Self-GPay</t>
+        </is>
+      </c>
+      <c r="Q506" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="n">
+        <v>504</v>
+      </c>
+      <c r="B507" s="127" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C507">
+        <f>IF(B507="","",TEXT(B507,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>Cement transport charge</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I507" t="n">
+        <v>1</v>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K507" t="n">
+        <v>300</v>
+      </c>
+      <c r="L507">
+        <f>IF(OR(I507="",K507=""),"",I507*K507)</f>
+        <v/>
+      </c>
+      <c r="N507">
+        <f>M507*L507</f>
+        <v/>
+      </c>
+      <c r="O507">
+        <f>IF(L507="","",IF(M507="",L507,L507*(1-M507)))</f>
+        <v/>
+      </c>
+      <c r="P507" t="inlineStr">
+        <is>
+          <t>Self-GPay</t>
+        </is>
+      </c>
+      <c r="Q507" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="n">
+        <v>505</v>
+      </c>
+      <c r="B508" s="127" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C508">
+        <f>IF(B508="","",TEXT(B508,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>Daily Labour-Unloading</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>Cement unloading labour</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I508" t="n">
+        <v>1</v>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K508" t="n">
+        <v>200</v>
+      </c>
+      <c r="L508">
+        <f>IF(OR(I508="",K508=""),"",I508*K508)</f>
+        <v/>
+      </c>
+      <c r="N508">
+        <f>M508*L508</f>
+        <v/>
+      </c>
+      <c r="O508">
+        <f>IF(L508="","",IF(M508="",L508,L508*(1-M508)))</f>
+        <v/>
+      </c>
+      <c r="P508" t="inlineStr">
+        <is>
+          <t>Self-GPay</t>
+        </is>
+      </c>
+      <c r="Q508" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B506" s="60" t="n"/>
-      <c r="C506" s="60" t="n"/>
-      <c r="D506" s="60" t="n"/>
-      <c r="E506" s="60" t="n"/>
-      <c r="F506" s="60" t="n"/>
-      <c r="G506" s="60" t="n"/>
-      <c r="H506" s="60" t="n"/>
-      <c r="I506" s="60" t="n"/>
-      <c r="J506" s="60" t="n"/>
-      <c r="K506" s="60" t="n"/>
-      <c r="L506" s="61">
-        <f>SUM(L5:L505)</f>
-        <v/>
-      </c>
-      <c r="M506" s="60" t="n"/>
-      <c r="N506" s="60" t="n"/>
-      <c r="O506" s="61">
-        <f>SUM(O5:O505)</f>
-        <v/>
-      </c>
-      <c r="P506" s="60" t="n"/>
-      <c r="Q506" s="60" t="n"/>
+      <c r="B509" s="60" t="n"/>
+      <c r="C509" s="60" t="n"/>
+      <c r="D509" s="60" t="n"/>
+      <c r="E509" s="60" t="n"/>
+      <c r="F509" s="60" t="n"/>
+      <c r="G509" s="60" t="n"/>
+      <c r="H509" s="60" t="n"/>
+      <c r="I509" s="60" t="n"/>
+      <c r="J509" s="60" t="n"/>
+      <c r="K509" s="60" t="n"/>
+      <c r="L509" s="61">
+        <f>SUM(L5:L508)</f>
+        <v/>
+      </c>
+      <c r="M509" s="60" t="n"/>
+      <c r="N509" s="60" t="n"/>
+      <c r="O509" s="61">
+        <f>SUM(O5:O508)</f>
+        <v/>
+      </c>
+      <c r="P509" s="60" t="n"/>
+      <c r="Q509" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -33633,18 +33839,51 @@
       <c r="M29" s="47" t="n"/>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="99">
-      <c r="A30" s="43" t="n"/>
-      <c r="B30" s="53" t="n"/>
-      <c r="C30" s="55" t="n"/>
-      <c r="D30" s="55" t="n"/>
-      <c r="E30" s="55" t="n"/>
-      <c r="F30" s="55" t="n"/>
-      <c r="G30" s="63" t="n"/>
-      <c r="H30" s="55" t="n"/>
+      <c r="A30" s="43" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="53" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C30" s="55" t="inlineStr">
+        <is>
+          <t>Self-GPay</t>
+        </is>
+      </c>
+      <c r="D30" s="55" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E30" s="55" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F30" s="55" t="inlineStr">
+        <is>
+          <t>Cement 50B + transport + labour</t>
+        </is>
+      </c>
+      <c r="G30" s="63" t="n">
+        <v>18500</v>
+      </c>
+      <c r="H30" s="55" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I30" s="55" t="n"/>
       <c r="J30" s="55" t="n"/>
-      <c r="K30" s="55" t="n"/>
-      <c r="L30" s="58" t="n"/>
+      <c r="K30" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L30" s="58">
+        <f>L29+G30</f>
+        <v/>
+      </c>
       <c r="M30" s="55" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="99">

</xml_diff>

<commit_message>
Update: Pappu Hardware Bill 4 settled — ₹1,300 paid by Self-GPay (21-Jun)
- Pappu Hardware status: 'due' → 'paid' (fully settled)
- Payment Tracker row 31: ₹1,300 GPay
- balanceDue: ₹14,000 → ₹12,700 (only Mukesh Yadav remaining)
- totalPaid: ₹14,56,797 → ₹14,58,097
- Removed Pappu from unpaid list

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -33887,18 +33887,51 @@
       <c r="M30" s="55" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="99">
-      <c r="A31" s="41" t="n"/>
-      <c r="B31" s="45" t="n"/>
-      <c r="C31" s="47" t="n"/>
-      <c r="D31" s="47" t="n"/>
-      <c r="E31" s="47" t="n"/>
-      <c r="F31" s="47" t="n"/>
-      <c r="G31" s="62" t="n"/>
-      <c r="H31" s="47" t="n"/>
+      <c r="A31" s="41" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="45" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C31" s="47" t="inlineStr">
+        <is>
+          <t>Self-GPay</t>
+        </is>
+      </c>
+      <c r="D31" s="47" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E31" s="47" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F31" s="47" t="inlineStr">
+        <is>
+          <t>Soft wire 10 Kg — Bill 4 settlement</t>
+        </is>
+      </c>
+      <c r="G31" s="62" t="n">
+        <v>1300</v>
+      </c>
+      <c r="H31" s="47" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I31" s="47" t="n"/>
       <c r="J31" s="47" t="n"/>
-      <c r="K31" s="47" t="n"/>
-      <c r="L31" s="50" t="n"/>
+      <c r="K31" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L31" s="50">
+        <f>L30+G31</f>
+        <v/>
+      </c>
       <c r="M31" s="47" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="99">

</xml_diff>

<commit_message>
Update: Brick tractor 13, Mukesh 22 trailers mitti, Labour 16100+2200, Papa ₹2000 payment (22-23 Jun)
All Transactions (4 new rows):
- Brick Company: tractor 13 — 1,500 bricks @ ₹8.5 = ₹12,750 (23-Jun)
- Mukesh Yadav: 22 trailers mitti @ ₹600 = ₹13,200 (22-Jun)
- Daily Labour: mitti bharai 46 labourers @ ₹350 = ₹16,100 (22-Jun)
- Daily Labour: kitchen area labour = ₹2,200 (23-Jun)

Payment Tracker: Papa ₹2,000 → Daily Labour (22-Jun)
Excel: 0 errors, 2750 formulas verified
vendors=categories=totalBilled=₹13,99,047 ✓

Updated totals:
- Total Billed: ₹12,54,797 → ₹13,99,047 (+₹44,250)
- Total Paid: ₹14,58,097 → ₹14,60,097 (+₹2,000)
- Total Due: ₹12,700 → ₹42,200 (Mukesh ₹25,900 + Labour ₹16,300)
- Bricks: 18,000 → 19,500 nos (13 tractors); credit left ₹2,03,250

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6451,7 +6451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q509"/>
+  <dimension ref="A1:Q513"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -20665,33 +20665,281 @@
       </c>
     </row>
     <row r="509">
-      <c r="A509" s="60" t="inlineStr">
+      <c r="A509" t="n">
+        <v>506</v>
+      </c>
+      <c r="B509" s="127" t="n">
+        <v>46196</v>
+      </c>
+      <c r="C509">
+        <f>IF(B509="","",TEXT(B509,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>Bricks</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>Brick delivery — tractor 13 (1,500 bricks @ ₹8.5)</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>Brick Company</t>
+        </is>
+      </c>
+      <c r="I509" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>Nos</t>
+        </is>
+      </c>
+      <c r="K509" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="L509">
+        <f>IF(OR(I509="",K509=""),"",I509*K509)</f>
+        <v/>
+      </c>
+      <c r="N509">
+        <f>M509*L509</f>
+        <v/>
+      </c>
+      <c r="O509">
+        <f>IF(L509="","",IF(M509="",L509,L509*(1-M509)))</f>
+        <v/>
+      </c>
+      <c r="P509" t="inlineStr"/>
+      <c r="Q509" t="inlineStr"/>
+    </row>
+    <row r="510">
+      <c r="A510" t="n">
+        <v>507</v>
+      </c>
+      <c r="B510" s="127" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C510">
+        <f>IF(B510="","",TEXT(B510,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>Land Development</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>Mitti filling 22 trailers @ ₹600</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="I510" t="n">
+        <v>22</v>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>Trailer</t>
+        </is>
+      </c>
+      <c r="K510" t="n">
+        <v>600</v>
+      </c>
+      <c r="L510">
+        <f>IF(OR(I510="",K510=""),"",I510*K510)</f>
+        <v/>
+      </c>
+      <c r="N510">
+        <f>M510*L510</f>
+        <v/>
+      </c>
+      <c r="O510">
+        <f>IF(L510="","",IF(M510="",L510,L510*(1-M510)))</f>
+        <v/>
+      </c>
+      <c r="P510" t="inlineStr"/>
+      <c r="Q510" t="inlineStr"/>
+    </row>
+    <row r="511">
+      <c r="A511" t="n">
+        <v>508</v>
+      </c>
+      <c r="B511" s="127" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C511">
+        <f>IF(B511="","",TEXT(B511,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>Daily Labour-Mitti Bharai</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>Mitti bharai 46 labourers @ ₹350</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>Daily Labour</t>
+        </is>
+      </c>
+      <c r="I511" t="n">
+        <v>46</v>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="K511" t="n">
+        <v>350</v>
+      </c>
+      <c r="L511">
+        <f>IF(OR(I511="",K511=""),"",I511*K511)</f>
+        <v/>
+      </c>
+      <c r="N511">
+        <f>M511*L511</f>
+        <v/>
+      </c>
+      <c r="O511">
+        <f>IF(L511="","",IF(M511="",L511,L511*(1-M511)))</f>
+        <v/>
+      </c>
+      <c r="P511" t="inlineStr"/>
+      <c r="Q511" t="inlineStr"/>
+    </row>
+    <row r="512">
+      <c r="A512" t="n">
+        <v>509</v>
+      </c>
+      <c r="B512" s="127" t="n">
+        <v>46196</v>
+      </c>
+      <c r="C512">
+        <f>IF(B512="","",TEXT(B512,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>Daily Labour-Kitchen</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>Kitchen area labour</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>Daily Labour</t>
+        </is>
+      </c>
+      <c r="I512" t="n">
+        <v>1</v>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K512" t="n">
+        <v>2200</v>
+      </c>
+      <c r="L512">
+        <f>IF(OR(I512="",K512=""),"",I512*K512)</f>
+        <v/>
+      </c>
+      <c r="N512">
+        <f>M512*L512</f>
+        <v/>
+      </c>
+      <c r="O512">
+        <f>IF(L512="","",IF(M512="",L512,L512*(1-M512)))</f>
+        <v/>
+      </c>
+      <c r="P512" t="inlineStr"/>
+      <c r="Q512" t="inlineStr"/>
+    </row>
+    <row r="513">
+      <c r="A513" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B509" s="60" t="n"/>
-      <c r="C509" s="60" t="n"/>
-      <c r="D509" s="60" t="n"/>
-      <c r="E509" s="60" t="n"/>
-      <c r="F509" s="60" t="n"/>
-      <c r="G509" s="60" t="n"/>
-      <c r="H509" s="60" t="n"/>
-      <c r="I509" s="60" t="n"/>
-      <c r="J509" s="60" t="n"/>
-      <c r="K509" s="60" t="n"/>
-      <c r="L509" s="61">
-        <f>SUM(L5:L508)</f>
-        <v/>
-      </c>
-      <c r="M509" s="60" t="n"/>
-      <c r="N509" s="60" t="n"/>
-      <c r="O509" s="61">
-        <f>SUM(O5:O508)</f>
-        <v/>
-      </c>
-      <c r="P509" s="60" t="n"/>
-      <c r="Q509" s="60" t="n"/>
+      <c r="B513" s="60" t="n"/>
+      <c r="C513" s="60" t="n"/>
+      <c r="D513" s="60" t="n"/>
+      <c r="E513" s="60" t="n"/>
+      <c r="F513" s="60" t="n"/>
+      <c r="G513" s="60" t="n"/>
+      <c r="H513" s="60" t="n"/>
+      <c r="I513" s="60" t="n"/>
+      <c r="J513" s="60" t="n"/>
+      <c r="K513" s="60" t="n"/>
+      <c r="L513" s="61">
+        <f>SUM(L5:L512)</f>
+        <v/>
+      </c>
+      <c r="M513" s="60" t="n"/>
+      <c r="N513" s="60" t="n"/>
+      <c r="O513" s="61">
+        <f>SUM(O5:O512)</f>
+        <v/>
+      </c>
+      <c r="P513" s="60" t="n"/>
+      <c r="Q513" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -33935,18 +34183,51 @@
       <c r="M31" s="47" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="99">
-      <c r="A32" s="43" t="n"/>
-      <c r="B32" s="53" t="n"/>
-      <c r="C32" s="55" t="n"/>
-      <c r="D32" s="55" t="n"/>
-      <c r="E32" s="55" t="n"/>
-      <c r="F32" s="55" t="n"/>
-      <c r="G32" s="63" t="n"/>
-      <c r="H32" s="55" t="n"/>
+      <c r="A32" s="43" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="53" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C32" s="55" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D32" s="55" t="inlineStr">
+        <is>
+          <t>Daily Labour</t>
+        </is>
+      </c>
+      <c r="E32" s="55" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F32" s="55" t="inlineStr">
+        <is>
+          <t>Mitti bharai labour payment</t>
+        </is>
+      </c>
+      <c r="G32" s="63" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H32" s="55" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I32" s="55" t="n"/>
       <c r="J32" s="55" t="n"/>
-      <c r="K32" s="55" t="n"/>
-      <c r="L32" s="58" t="n"/>
+      <c r="K32" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L32" s="58">
+        <f>L31+G32</f>
+        <v/>
+      </c>
       <c r="M32" s="55" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="99">

</xml_diff>

<commit_message>
Update: All labour payment done by Papa — ₹16,300 (23-Jun)
Daily Labour fully settled (billed = paid = ₹51,375)
Payment Tracker row 33: Papa ₹16,300 GPay
- balanceDue: ₹42,200 → ₹25,900 (only Mukesh Yadav remaining)
- totalPaid: ₹14,60,097 → ₹14,76,397
- Papa total: ₹2,47,135 → ₹2,63,435 (17.8%)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -20723,8 +20723,6 @@
         <f>IF(L509="","",IF(M509="",L509,L509*(1-M509)))</f>
         <v/>
       </c>
-      <c r="P509" t="inlineStr"/>
-      <c r="Q509" t="inlineStr"/>
     </row>
     <row r="510">
       <c r="A510" t="n">
@@ -20785,8 +20783,6 @@
         <f>IF(L510="","",IF(M510="",L510,L510*(1-M510)))</f>
         <v/>
       </c>
-      <c r="P510" t="inlineStr"/>
-      <c r="Q510" t="inlineStr"/>
     </row>
     <row r="511">
       <c r="A511" t="n">
@@ -20847,8 +20843,6 @@
         <f>IF(L511="","",IF(M511="",L511,L511*(1-M511)))</f>
         <v/>
       </c>
-      <c r="P511" t="inlineStr"/>
-      <c r="Q511" t="inlineStr"/>
     </row>
     <row r="512">
       <c r="A512" t="n">
@@ -20909,8 +20903,6 @@
         <f>IF(L512="","",IF(M512="",L512,L512*(1-M512)))</f>
         <v/>
       </c>
-      <c r="P512" t="inlineStr"/>
-      <c r="Q512" t="inlineStr"/>
     </row>
     <row r="513">
       <c r="A513" s="60" t="inlineStr">
@@ -34231,18 +34223,51 @@
       <c r="M32" s="55" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="99">
-      <c r="A33" s="41" t="n"/>
-      <c r="B33" s="45" t="n"/>
-      <c r="C33" s="47" t="n"/>
-      <c r="D33" s="47" t="n"/>
-      <c r="E33" s="47" t="n"/>
-      <c r="F33" s="47" t="n"/>
-      <c r="G33" s="62" t="n"/>
-      <c r="H33" s="47" t="n"/>
+      <c r="A33" s="41" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="45" t="n">
+        <v>46196</v>
+      </c>
+      <c r="C33" s="47" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="inlineStr">
+        <is>
+          <t>Daily Labour</t>
+        </is>
+      </c>
+      <c r="E33" s="47" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F33" s="47" t="inlineStr">
+        <is>
+          <t>Full labour settlement — mitti bharai + kitchen</t>
+        </is>
+      </c>
+      <c r="G33" s="62" t="n">
+        <v>16300</v>
+      </c>
+      <c r="H33" s="47" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I33" s="47" t="n"/>
       <c r="J33" s="47" t="n"/>
-      <c r="K33" s="47" t="n"/>
-      <c r="L33" s="50" t="n"/>
+      <c r="K33" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L33" s="50">
+        <f>L32+G33</f>
+        <v/>
+      </c>
       <c r="M33" s="47" t="n"/>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="99">

</xml_diff>

<commit_message>
Update: Mukesh Yadav 20 trailers mitti (23-Jun, unpaid) — ₹12,000
All Transactions row 513: 20 trailers @ ₹600 = ₹12,000
No payment — balance due increases.
Excel: 0 errors, 2755 formulas verified.
totalBilled=vendors=categories=₹13,11,047 ✓

Updated totals:
- Total Billed: ₹12,99,047 → ₹13,11,047 (+₹12,000)
- Mukesh Yadav: ₹89,100 → ₹1,01,100 billed; due ₹37,900
- Land Development: 104 → 124 trailers; ₹62,400 → ₹74,400
- Jun-2026: ₹4,69,455 → ₹4,81,455

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6451,7 +6451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q513"/>
+  <dimension ref="A1:Q514"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -20905,33 +20905,95 @@
       </c>
     </row>
     <row r="513">
-      <c r="A513" s="60" t="inlineStr">
+      <c r="A513" t="n">
+        <v>510</v>
+      </c>
+      <c r="B513" s="127" t="n">
+        <v>46196</v>
+      </c>
+      <c r="C513">
+        <f>IF(B513="","",TEXT(B513,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Land Development</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>Mitti filling 20 trailers @ ₹600</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="I513" t="n">
+        <v>20</v>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>Trailer</t>
+        </is>
+      </c>
+      <c r="K513" t="n">
+        <v>600</v>
+      </c>
+      <c r="L513">
+        <f>IF(OR(I513="",K513=""),"",I513*K513)</f>
+        <v/>
+      </c>
+      <c r="N513">
+        <f>M513*L513</f>
+        <v/>
+      </c>
+      <c r="O513">
+        <f>IF(L513="","",IF(M513="",L513,L513*(1-M513)))</f>
+        <v/>
+      </c>
+      <c r="P513" t="inlineStr"/>
+      <c r="Q513" t="inlineStr"/>
+    </row>
+    <row r="514">
+      <c r="A514" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B513" s="60" t="n"/>
-      <c r="C513" s="60" t="n"/>
-      <c r="D513" s="60" t="n"/>
-      <c r="E513" s="60" t="n"/>
-      <c r="F513" s="60" t="n"/>
-      <c r="G513" s="60" t="n"/>
-      <c r="H513" s="60" t="n"/>
-      <c r="I513" s="60" t="n"/>
-      <c r="J513" s="60" t="n"/>
-      <c r="K513" s="60" t="n"/>
-      <c r="L513" s="61">
-        <f>SUM(L5:L512)</f>
-        <v/>
-      </c>
-      <c r="M513" s="60" t="n"/>
-      <c r="N513" s="60" t="n"/>
-      <c r="O513" s="61">
-        <f>SUM(O5:O512)</f>
-        <v/>
-      </c>
-      <c r="P513" s="60" t="n"/>
-      <c r="Q513" s="60" t="n"/>
+      <c r="B514" s="60" t="n"/>
+      <c r="C514" s="60" t="n"/>
+      <c r="D514" s="60" t="n"/>
+      <c r="E514" s="60" t="n"/>
+      <c r="F514" s="60" t="n"/>
+      <c r="G514" s="60" t="n"/>
+      <c r="H514" s="60" t="n"/>
+      <c r="I514" s="60" t="n"/>
+      <c r="J514" s="60" t="n"/>
+      <c r="K514" s="60" t="n"/>
+      <c r="L514" s="61">
+        <f>SUM(L5:L513)</f>
+        <v/>
+      </c>
+      <c r="M514" s="60" t="n"/>
+      <c r="N514" s="60" t="n"/>
+      <c r="O514" s="61">
+        <f>SUM(O5:O513)</f>
+        <v/>
+      </c>
+      <c r="P514" s="60" t="n"/>
+      <c r="Q514" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>

</xml_diff>

<commit_message>
Update: JCB 1.25 hrs (4-Jul) + ₹30,000 payment to Mukesh Yadav (5-Jul)
All Transactions row 514: JCB 1.25 hrs @ ₹1,000 = ₹1,250
Payment Tracker row 34: Self-GPay ₹30,000 to Mukesh Yadav
Excel: 0 errors, 2760 formulas verified.

Mukesh Yadav: billed ₹1,01,100→₹1,02,350; paid ₹63,200→₹93,200; due ₹37,900→₹9,150
totalBilled=vendors=categories=monthly=₹13,12,297 ✓
totalPaid=payers=₹15,06,397 ✓

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6451,7 +6451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q514"/>
+  <dimension ref="A1:Q515"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -20963,37 +20963,95 @@
         <f>IF(L513="","",IF(M513="",L513,L513*(1-M513)))</f>
         <v/>
       </c>
-      <c r="P513" t="inlineStr"/>
-      <c r="Q513" t="inlineStr"/>
     </row>
     <row r="514">
-      <c r="A514" s="60" t="inlineStr">
+      <c r="A514" t="n">
+        <v>511</v>
+      </c>
+      <c r="B514" s="127" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C514">
+        <f>IF(B514="","",TEXT(B514,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>Land Development</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>JCB Work</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>JCB work 1.25 hrs @ ₹1,000</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="I514" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>Hour</t>
+        </is>
+      </c>
+      <c r="K514" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L514">
+        <f>IF(OR(I514="",K514=""),"",I514*K514)</f>
+        <v/>
+      </c>
+      <c r="N514">
+        <f>M514*L514</f>
+        <v/>
+      </c>
+      <c r="O514">
+        <f>IF(L514="","",IF(M514="",L514,L514*(1-M514)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B514" s="60" t="n"/>
-      <c r="C514" s="60" t="n"/>
-      <c r="D514" s="60" t="n"/>
-      <c r="E514" s="60" t="n"/>
-      <c r="F514" s="60" t="n"/>
-      <c r="G514" s="60" t="n"/>
-      <c r="H514" s="60" t="n"/>
-      <c r="I514" s="60" t="n"/>
-      <c r="J514" s="60" t="n"/>
-      <c r="K514" s="60" t="n"/>
-      <c r="L514" s="61">
-        <f>SUM(L5:L513)</f>
-        <v/>
-      </c>
-      <c r="M514" s="60" t="n"/>
-      <c r="N514" s="60" t="n"/>
-      <c r="O514" s="61">
-        <f>SUM(O5:O513)</f>
-        <v/>
-      </c>
-      <c r="P514" s="60" t="n"/>
-      <c r="Q514" s="60" t="n"/>
+      <c r="B515" s="60" t="n"/>
+      <c r="C515" s="60" t="n"/>
+      <c r="D515" s="60" t="n"/>
+      <c r="E515" s="60" t="n"/>
+      <c r="F515" s="60" t="n"/>
+      <c r="G515" s="60" t="n"/>
+      <c r="H515" s="60" t="n"/>
+      <c r="I515" s="60" t="n"/>
+      <c r="J515" s="60" t="n"/>
+      <c r="K515" s="60" t="n"/>
+      <c r="L515" s="61">
+        <f>SUM(L5:L514)</f>
+        <v/>
+      </c>
+      <c r="M515" s="60" t="n"/>
+      <c r="N515" s="60" t="n"/>
+      <c r="O515" s="61">
+        <f>SUM(O5:O514)</f>
+        <v/>
+      </c>
+      <c r="P515" s="60" t="n"/>
+      <c r="Q515" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -34333,18 +34391,51 @@
       <c r="M33" s="47" t="n"/>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="99">
-      <c r="A34" s="43" t="n"/>
-      <c r="B34" s="53" t="n"/>
-      <c r="C34" s="55" t="n"/>
-      <c r="D34" s="55" t="n"/>
-      <c r="E34" s="55" t="n"/>
-      <c r="F34" s="55" t="n"/>
-      <c r="G34" s="63" t="n"/>
-      <c r="H34" s="55" t="n"/>
+      <c r="A34" s="43" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="53" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C34" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D34" s="55" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="E34" s="55" t="inlineStr">
+        <is>
+          <t>Land Development</t>
+        </is>
+      </c>
+      <c r="F34" s="55" t="inlineStr">
+        <is>
+          <t>Mitti + JCB balance payment</t>
+        </is>
+      </c>
+      <c r="G34" s="63" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H34" s="55" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I34" s="55" t="n"/>
       <c r="J34" s="55" t="n"/>
-      <c r="K34" s="55" t="n"/>
-      <c r="L34" s="58" t="n"/>
+      <c r="K34" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L34" s="58">
+        <f>L33+G34</f>
+        <v/>
+      </c>
       <c r="M34" s="55" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="99">

</xml_diff>

<commit_message>
Update: Econ Builder ₹5,000 (Papa 22-Jun) + ₹75,000 (Self 5-Jul) engineer fees
All Transactions rows 515-516: Professional Fees — Econ Builder
Payment Tracker rows 35-36: Papa GPay ₹5,000 + Self GPay ₹75,000
Excel: 0 errors, 2768 formulas verified.

Econ Builder: billed ₹2,26,000→₹3,06,000; paid ₹2,26,000→₹3,06,000 (settled)
totalBilled=vendors=categories=monthly=₹13,92,297 ✓
totalPaid=payers=₹15,86,397 ✓

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6451,7 +6451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q515"/>
+  <dimension ref="A1:Q517"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -21025,33 +21025,165 @@
       </c>
     </row>
     <row r="515">
-      <c r="A515" s="60" t="inlineStr">
+      <c r="A515" t="n">
+        <v>512</v>
+      </c>
+      <c r="B515" s="127" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C515">
+        <f>IF(B515="","",TEXT(B515,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>Engineer Supervision</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>Engineer supervision fee — Jun payment</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I515" t="n">
+        <v>1</v>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K515" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L515">
+        <f>IF(OR(I515="",K515=""),"",I515*K515)</f>
+        <v/>
+      </c>
+      <c r="O515">
+        <f>IF(L515="","",IF(M515="",L515,L515*(1-M515)))</f>
+        <v/>
+      </c>
+      <c r="P515" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="Q515" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="n">
+        <v>513</v>
+      </c>
+      <c r="B516" s="127" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C516">
+        <f>IF(B516="","",TEXT(B516,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>Engineer Supervision</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>Engineer supervision fee — Jul payment</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I516" t="n">
+        <v>1</v>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K516" t="n">
+        <v>75000</v>
+      </c>
+      <c r="L516">
+        <f>IF(OR(I516="",K516=""),"",I516*K516)</f>
+        <v/>
+      </c>
+      <c r="O516">
+        <f>IF(L516="","",IF(M516="",L516,L516*(1-M516)))</f>
+        <v/>
+      </c>
+      <c r="P516" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="Q516" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B515" s="60" t="n"/>
-      <c r="C515" s="60" t="n"/>
-      <c r="D515" s="60" t="n"/>
-      <c r="E515" s="60" t="n"/>
-      <c r="F515" s="60" t="n"/>
-      <c r="G515" s="60" t="n"/>
-      <c r="H515" s="60" t="n"/>
-      <c r="I515" s="60" t="n"/>
-      <c r="J515" s="60" t="n"/>
-      <c r="K515" s="60" t="n"/>
-      <c r="L515" s="61">
-        <f>SUM(L5:L514)</f>
-        <v/>
-      </c>
-      <c r="M515" s="60" t="n"/>
-      <c r="N515" s="60" t="n"/>
-      <c r="O515" s="61">
-        <f>SUM(O5:O514)</f>
-        <v/>
-      </c>
-      <c r="P515" s="60" t="n"/>
-      <c r="Q515" s="60" t="n"/>
+      <c r="B517" s="60" t="n"/>
+      <c r="C517" s="60" t="n"/>
+      <c r="D517" s="60" t="n"/>
+      <c r="E517" s="60" t="n"/>
+      <c r="F517" s="60" t="n"/>
+      <c r="G517" s="60" t="n"/>
+      <c r="H517" s="60" t="n"/>
+      <c r="I517" s="60" t="n"/>
+      <c r="J517" s="60" t="n"/>
+      <c r="K517" s="60" t="n"/>
+      <c r="L517" s="61">
+        <f>SUM(L5:L516)</f>
+        <v/>
+      </c>
+      <c r="M517" s="60" t="n"/>
+      <c r="N517" s="60" t="n"/>
+      <c r="O517" s="61">
+        <f>SUM(O5:O516)</f>
+        <v/>
+      </c>
+      <c r="P517" s="60" t="n"/>
+      <c r="Q517" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -34439,33 +34571,99 @@
       <c r="M34" s="55" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="99">
-      <c r="A35" s="41" t="n"/>
-      <c r="B35" s="45" t="n"/>
-      <c r="C35" s="47" t="n"/>
-      <c r="D35" s="47" t="n"/>
-      <c r="E35" s="47" t="n"/>
-      <c r="F35" s="47" t="n"/>
-      <c r="G35" s="62" t="n"/>
-      <c r="H35" s="47" t="n"/>
+      <c r="A35" s="41" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="45" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C35" s="47" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D35" s="47" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E35" s="47" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F35" s="47" t="inlineStr">
+        <is>
+          <t>Engineer supervision fee — Jun payment</t>
+        </is>
+      </c>
+      <c r="G35" s="62" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H35" s="47" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I35" s="47" t="n"/>
       <c r="J35" s="47" t="n"/>
-      <c r="K35" s="47" t="n"/>
-      <c r="L35" s="50" t="n"/>
+      <c r="K35" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L35" s="50">
+        <f>L34+G35</f>
+        <v/>
+      </c>
       <c r="M35" s="47" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="99">
-      <c r="A36" s="43" t="n"/>
-      <c r="B36" s="53" t="n"/>
-      <c r="C36" s="55" t="n"/>
-      <c r="D36" s="55" t="n"/>
-      <c r="E36" s="55" t="n"/>
-      <c r="F36" s="55" t="n"/>
-      <c r="G36" s="63" t="n"/>
-      <c r="H36" s="55" t="n"/>
+      <c r="A36" s="43" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="53" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C36" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D36" s="55" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E36" s="55" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F36" s="55" t="inlineStr">
+        <is>
+          <t>Engineer supervision fee — Jul payment</t>
+        </is>
+      </c>
+      <c r="G36" s="63" t="n">
+        <v>75000</v>
+      </c>
+      <c r="H36" s="55" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I36" s="55" t="n"/>
       <c r="J36" s="55" t="n"/>
-      <c r="K36" s="55" t="n"/>
-      <c r="L36" s="58" t="n"/>
+      <c r="K36" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L36" s="58">
+        <f>L35+G36</f>
+        <v/>
+      </c>
       <c r="M36" s="55" t="n"/>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="99">

</xml_diff>

<commit_message>
Update: Sand Truck 3 — 944 CFT ₹56,500 (Self ₹46,500 + Papa ₹10,000) — 5-Jul
All Transactions row 517: Sand 944 CFT @ ₹59.85/CFT = ₹56,500
Payment Tracker rows 37-38: Self GPay ₹46,500 + Papa GPay ₹10,000
Excel: 0 errors, 2773 formulas verified.

Sand Truck Wala: ₹1,10,000 → ₹1,66,500 (3 trucks, 2,782 CFT total)
Building Materials: ₹5,59,832 → ₹6,16,332
totalBilled=vendors=categories=monthly=₹14,48,797 ✓
totalPaid=payers=₹16,42,897 ✓

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6451,7 +6451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q517"/>
+  <dimension ref="A1:Q518"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -21157,33 +21157,89 @@
       </c>
     </row>
     <row r="517">
-      <c r="A517" s="60" t="inlineStr">
+      <c r="A517" t="n">
+        <v>514</v>
+      </c>
+      <c r="B517" s="127" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C517">
+        <f>IF(B517="","",TEXT(B517,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>Sand</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>Sand Truck 3 — 944 CFT @ ₹59.85/CFT</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>Sand Truck Wala</t>
+        </is>
+      </c>
+      <c r="I517" t="n">
+        <v>1</v>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K517" t="n">
+        <v>56500</v>
+      </c>
+      <c r="L517">
+        <f>IF(OR(I517="",K517=""),"",I517*K517)</f>
+        <v/>
+      </c>
+      <c r="O517">
+        <f>IF(L517="","",IF(M517="",L517,L517*(1-M517)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B517" s="60" t="n"/>
-      <c r="C517" s="60" t="n"/>
-      <c r="D517" s="60" t="n"/>
-      <c r="E517" s="60" t="n"/>
-      <c r="F517" s="60" t="n"/>
-      <c r="G517" s="60" t="n"/>
-      <c r="H517" s="60" t="n"/>
-      <c r="I517" s="60" t="n"/>
-      <c r="J517" s="60" t="n"/>
-      <c r="K517" s="60" t="n"/>
-      <c r="L517" s="61">
-        <f>SUM(L5:L516)</f>
-        <v/>
-      </c>
-      <c r="M517" s="60" t="n"/>
-      <c r="N517" s="60" t="n"/>
-      <c r="O517" s="61">
-        <f>SUM(O5:O516)</f>
-        <v/>
-      </c>
-      <c r="P517" s="60" t="n"/>
-      <c r="Q517" s="60" t="n"/>
+      <c r="B518" s="60" t="n"/>
+      <c r="C518" s="60" t="n"/>
+      <c r="D518" s="60" t="n"/>
+      <c r="E518" s="60" t="n"/>
+      <c r="F518" s="60" t="n"/>
+      <c r="G518" s="60" t="n"/>
+      <c r="H518" s="60" t="n"/>
+      <c r="I518" s="60" t="n"/>
+      <c r="J518" s="60" t="n"/>
+      <c r="K518" s="60" t="n"/>
+      <c r="L518" s="61">
+        <f>SUM(L5:L517)</f>
+        <v/>
+      </c>
+      <c r="M518" s="60" t="n"/>
+      <c r="N518" s="60" t="n"/>
+      <c r="O518" s="61">
+        <f>SUM(O5:O517)</f>
+        <v/>
+      </c>
+      <c r="P518" s="60" t="n"/>
+      <c r="Q518" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -34667,33 +34723,99 @@
       <c r="M36" s="55" t="n"/>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="99">
-      <c r="A37" s="41" t="n"/>
-      <c r="B37" s="45" t="n"/>
-      <c r="C37" s="47" t="n"/>
-      <c r="D37" s="47" t="n"/>
-      <c r="E37" s="47" t="n"/>
-      <c r="F37" s="47" t="n"/>
-      <c r="G37" s="62" t="n"/>
-      <c r="H37" s="47" t="n"/>
+      <c r="A37" s="41" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="45" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C37" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D37" s="47" t="inlineStr">
+        <is>
+          <t>Sand Truck Wala</t>
+        </is>
+      </c>
+      <c r="E37" s="47" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F37" s="47" t="inlineStr">
+        <is>
+          <t>Sand Truck 3 — 944 CFT</t>
+        </is>
+      </c>
+      <c r="G37" s="62" t="n">
+        <v>46500</v>
+      </c>
+      <c r="H37" s="47" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I37" s="47" t="n"/>
       <c r="J37" s="47" t="n"/>
-      <c r="K37" s="47" t="n"/>
-      <c r="L37" s="50" t="n"/>
+      <c r="K37" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L37" s="50">
+        <f>L36+G37</f>
+        <v/>
+      </c>
       <c r="M37" s="47" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="99">
-      <c r="A38" s="43" t="n"/>
-      <c r="B38" s="53" t="n"/>
-      <c r="C38" s="55" t="n"/>
-      <c r="D38" s="55" t="n"/>
-      <c r="E38" s="55" t="n"/>
-      <c r="F38" s="55" t="n"/>
-      <c r="G38" s="63" t="n"/>
-      <c r="H38" s="55" t="n"/>
+      <c r="A38" s="43" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="53" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C38" s="55" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D38" s="55" t="inlineStr">
+        <is>
+          <t>Sand Truck Wala</t>
+        </is>
+      </c>
+      <c r="E38" s="55" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F38" s="55" t="inlineStr">
+        <is>
+          <t>Sand Truck 3 — 944 CFT</t>
+        </is>
+      </c>
+      <c r="G38" s="63" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H38" s="55" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I38" s="55" t="n"/>
       <c r="J38" s="55" t="n"/>
-      <c r="K38" s="55" t="n"/>
-      <c r="L38" s="58" t="n"/>
+      <c r="K38" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L38" s="58">
+        <f>L37+G38</f>
+        <v/>
+      </c>
       <c r="M38" s="55" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="99">

</xml_diff>

<commit_message>
Update: Sand Truck 4 — 936 CFT ₹56,000 (Self) — 5-Jul
All Transactions row 518: Sand 936 CFT lumpsum ₹56,000
Payment Tracker row 39: Self GPay ₹56,000
Excel: 0 errors, 2777 formulas verified.

Sand Truck Wala: ₹1,66,500→₹2,22,500 (4 trucks, 3,718 CFT total)
Building Materials: ₹6,16,332→₹6,72,332
totalBilled=vendors=categories=monthly=₹15,04,797 ✓
totalPaid=payers=₹16,98,897 ✓

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6451,7 +6451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q518"/>
+  <dimension ref="A1:Q519"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -21213,33 +21213,99 @@
       </c>
     </row>
     <row r="518">
-      <c r="A518" s="60" t="inlineStr">
+      <c r="A518" t="n">
+        <v>515</v>
+      </c>
+      <c r="B518" s="127" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C518">
+        <f>IF(B518="","",TEXT(B518,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>Sand</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>Sand Truck 4 — 936 CFT @ ₹59.85/CFT</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>Sand Truck Wala</t>
+        </is>
+      </c>
+      <c r="I518" t="n">
+        <v>1</v>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K518" t="n">
+        <v>56000</v>
+      </c>
+      <c r="L518">
+        <f>IF(OR(I518="",K518=""),"",I518*K518)</f>
+        <v/>
+      </c>
+      <c r="O518">
+        <f>IF(L518="","",IF(M518="",L518,L518*(1-M518)))</f>
+        <v/>
+      </c>
+      <c r="P518" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="Q518" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B518" s="60" t="n"/>
-      <c r="C518" s="60" t="n"/>
-      <c r="D518" s="60" t="n"/>
-      <c r="E518" s="60" t="n"/>
-      <c r="F518" s="60" t="n"/>
-      <c r="G518" s="60" t="n"/>
-      <c r="H518" s="60" t="n"/>
-      <c r="I518" s="60" t="n"/>
-      <c r="J518" s="60" t="n"/>
-      <c r="K518" s="60" t="n"/>
-      <c r="L518" s="61">
-        <f>SUM(L5:L517)</f>
-        <v/>
-      </c>
-      <c r="M518" s="60" t="n"/>
-      <c r="N518" s="60" t="n"/>
-      <c r="O518" s="61">
-        <f>SUM(O5:O517)</f>
-        <v/>
-      </c>
-      <c r="P518" s="60" t="n"/>
-      <c r="Q518" s="60" t="n"/>
+      <c r="B519" s="60" t="n"/>
+      <c r="C519" s="60" t="n"/>
+      <c r="D519" s="60" t="n"/>
+      <c r="E519" s="60" t="n"/>
+      <c r="F519" s="60" t="n"/>
+      <c r="G519" s="60" t="n"/>
+      <c r="H519" s="60" t="n"/>
+      <c r="I519" s="60" t="n"/>
+      <c r="J519" s="60" t="n"/>
+      <c r="K519" s="60" t="n"/>
+      <c r="L519" s="61">
+        <f>SUM(L5:L518)</f>
+        <v/>
+      </c>
+      <c r="M519" s="60" t="n"/>
+      <c r="N519" s="60" t="n"/>
+      <c r="O519" s="61">
+        <f>SUM(O5:O518)</f>
+        <v/>
+      </c>
+      <c r="P519" s="60" t="n"/>
+      <c r="Q519" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -34819,18 +34885,51 @@
       <c r="M38" s="55" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="99">
-      <c r="A39" s="41" t="n"/>
-      <c r="B39" s="45" t="n"/>
-      <c r="C39" s="47" t="n"/>
-      <c r="D39" s="47" t="n"/>
-      <c r="E39" s="47" t="n"/>
-      <c r="F39" s="47" t="n"/>
-      <c r="G39" s="62" t="n"/>
-      <c r="H39" s="47" t="n"/>
+      <c r="A39" s="41" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="45" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C39" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D39" s="47" t="inlineStr">
+        <is>
+          <t>Sand Truck Wala</t>
+        </is>
+      </c>
+      <c r="E39" s="47" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F39" s="47" t="inlineStr">
+        <is>
+          <t>Sand Truck 4 — 936 CFT</t>
+        </is>
+      </c>
+      <c r="G39" s="62" t="n">
+        <v>56000</v>
+      </c>
+      <c r="H39" s="47" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I39" s="47" t="n"/>
       <c r="J39" s="47" t="n"/>
-      <c r="K39" s="47" t="n"/>
-      <c r="L39" s="50" t="n"/>
+      <c r="K39" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L39" s="50">
+        <f>L38+G39</f>
+        <v/>
+      </c>
       <c r="M39" s="47" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="99">

</xml_diff>

<commit_message>
Add Babloo Hardware bill ₹41,650 (Self, 5-Jul) — Cement+Steel+Gitti+DrFixit+Labour
All Transactions rows 519-524: 6 line items (Babloo Hardware)
  - Ultratech Super 30B @ ₹350 = ₹10,500
  - Ultratech PPC 30B @ ₹330 = ₹9,900
  - 6mm Tiscon 50pcs @ ₹228 = ₹11,400
  - Gitti 1 trailer = ₹7,500
  - Dr Fixit 10L = ₹1,400
  - Labour/unloading = ₹950
Payment Tracker row 40: Self GPay ₹41,650
Excel: 0 errors, 2796 formulas verified.

New vendor: Babloo Hardware (11th vendor)
totalBilled=vendors=categories=monthly=₹15,46,447 ✓
totalPaid=payers=₹17,40,547 ✓

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6451,7 +6451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q519"/>
+  <dimension ref="A1:Q525"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -21279,33 +21279,429 @@
       </c>
     </row>
     <row r="519">
-      <c r="A519" s="60" t="inlineStr">
+      <c r="A519" t="n">
+        <v>516</v>
+      </c>
+      <c r="B519" s="127" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C519">
+        <f>IF(B519="","",TEXT(B519,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>Ultratech Super Cement 30B @ ₹350</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>Babloo Hardware</t>
+        </is>
+      </c>
+      <c r="I519" t="n">
+        <v>30</v>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K519" t="n">
+        <v>350</v>
+      </c>
+      <c r="L519">
+        <f>IF(OR(I519="",K519=""),"",I519*K519)</f>
+        <v/>
+      </c>
+      <c r="O519">
+        <f>IF(L519="","",IF(M519="",L519,L519*(1-M519)))</f>
+        <v/>
+      </c>
+      <c r="P519" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="Q519" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="n">
+        <v>517</v>
+      </c>
+      <c r="B520" s="127" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C520">
+        <f>IF(B520="","",TEXT(B520,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>Ultratech Cement (PPC) 30B @ ₹330</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>Babloo Hardware</t>
+        </is>
+      </c>
+      <c r="I520" t="n">
+        <v>30</v>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K520" t="n">
+        <v>330</v>
+      </c>
+      <c r="L520">
+        <f>IF(OR(I520="",K520=""),"",I520*K520)</f>
+        <v/>
+      </c>
+      <c r="O520">
+        <f>IF(L520="","",IF(M520="",L520,L520*(1-M520)))</f>
+        <v/>
+      </c>
+      <c r="P520" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="Q520" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="n">
+        <v>518</v>
+      </c>
+      <c r="B521" s="127" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C521">
+        <f>IF(B521="","",TEXT(B521,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>Tiscon 6mm</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>6mm Tiscon Rod 50 pcs @ ₹228</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>Babloo Hardware</t>
+        </is>
+      </c>
+      <c r="I521" t="n">
+        <v>50</v>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>Pcs</t>
+        </is>
+      </c>
+      <c r="K521" t="n">
+        <v>228</v>
+      </c>
+      <c r="L521">
+        <f>IF(OR(I521="",K521=""),"",I521*K521)</f>
+        <v/>
+      </c>
+      <c r="O521">
+        <f>IF(L521="","",IF(M521="",L521,L521*(1-M521)))</f>
+        <v/>
+      </c>
+      <c r="P521" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="Q521" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="n">
+        <v>519</v>
+      </c>
+      <c r="B522" s="127" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C522">
+        <f>IF(B522="","",TEXT(B522,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>Concrete/Gitti</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>Gitti 1 trailer @ ₹7,500</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>Babloo Hardware</t>
+        </is>
+      </c>
+      <c r="I522" t="n">
+        <v>1</v>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>Trailer</t>
+        </is>
+      </c>
+      <c r="K522" t="n">
+        <v>7500</v>
+      </c>
+      <c r="L522">
+        <f>IF(OR(I522="",K522=""),"",I522*K522)</f>
+        <v/>
+      </c>
+      <c r="O522">
+        <f>IF(L522="","",IF(M522="",L522,L522*(1-M522)))</f>
+        <v/>
+      </c>
+      <c r="P522" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="Q522" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="n">
+        <v>520</v>
+      </c>
+      <c r="B523" s="127" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C523">
+        <f>IF(B523="","",TEXT(B523,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>Chemical</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>Dr Fixit 10 Litre @ ₹140</t>
+        </is>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>Babloo Hardware</t>
+        </is>
+      </c>
+      <c r="I523" t="n">
+        <v>10</v>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>Litre</t>
+        </is>
+      </c>
+      <c r="K523" t="n">
+        <v>140</v>
+      </c>
+      <c r="L523">
+        <f>IF(OR(I523="",K523=""),"",I523*K523)</f>
+        <v/>
+      </c>
+      <c r="O523">
+        <f>IF(L523="","",IF(M523="",L523,L523*(1-M523)))</f>
+        <v/>
+      </c>
+      <c r="P523" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="Q523" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="n">
+        <v>521</v>
+      </c>
+      <c r="B524" s="127" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C524">
+        <f>IF(B524="","",TEXT(B524,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>Labour/unloading charges</t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>Babloo Hardware</t>
+        </is>
+      </c>
+      <c r="I524" t="n">
+        <v>1</v>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K524" t="n">
+        <v>950</v>
+      </c>
+      <c r="L524">
+        <f>IF(OR(I524="",K524=""),"",I524*K524)</f>
+        <v/>
+      </c>
+      <c r="O524">
+        <f>IF(L524="","",IF(M524="",L524,L524*(1-M524)))</f>
+        <v/>
+      </c>
+      <c r="P524" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="Q524" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B519" s="60" t="n"/>
-      <c r="C519" s="60" t="n"/>
-      <c r="D519" s="60" t="n"/>
-      <c r="E519" s="60" t="n"/>
-      <c r="F519" s="60" t="n"/>
-      <c r="G519" s="60" t="n"/>
-      <c r="H519" s="60" t="n"/>
-      <c r="I519" s="60" t="n"/>
-      <c r="J519" s="60" t="n"/>
-      <c r="K519" s="60" t="n"/>
-      <c r="L519" s="61">
-        <f>SUM(L5:L518)</f>
-        <v/>
-      </c>
-      <c r="M519" s="60" t="n"/>
-      <c r="N519" s="60" t="n"/>
-      <c r="O519" s="61">
-        <f>SUM(O5:O518)</f>
-        <v/>
-      </c>
-      <c r="P519" s="60" t="n"/>
-      <c r="Q519" s="60" t="n"/>
+      <c r="B525" s="60" t="n"/>
+      <c r="C525" s="60" t="n"/>
+      <c r="D525" s="60" t="n"/>
+      <c r="E525" s="60" t="n"/>
+      <c r="F525" s="60" t="n"/>
+      <c r="G525" s="60" t="n"/>
+      <c r="H525" s="60" t="n"/>
+      <c r="I525" s="60" t="n"/>
+      <c r="J525" s="60" t="n"/>
+      <c r="K525" s="60" t="n"/>
+      <c r="L525" s="61">
+        <f>SUM(L5:L524)</f>
+        <v/>
+      </c>
+      <c r="M525" s="60" t="n"/>
+      <c r="N525" s="60" t="n"/>
+      <c r="O525" s="61">
+        <f>SUM(O5:O524)</f>
+        <v/>
+      </c>
+      <c r="P525" s="60" t="n"/>
+      <c r="Q525" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -34933,18 +35329,51 @@
       <c r="M39" s="47" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="99">
-      <c r="A40" s="43" t="n"/>
-      <c r="B40" s="53" t="n"/>
-      <c r="C40" s="55" t="n"/>
-      <c r="D40" s="55" t="n"/>
-      <c r="E40" s="55" t="n"/>
-      <c r="F40" s="55" t="n"/>
-      <c r="G40" s="63" t="n"/>
-      <c r="H40" s="55" t="n"/>
+      <c r="A40" s="43" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="53" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C40" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D40" s="55" t="inlineStr">
+        <is>
+          <t>Babloo Hardware</t>
+        </is>
+      </c>
+      <c r="E40" s="55" t="inlineStr">
+        <is>
+          <t>Building Materials + Steel + Labour</t>
+        </is>
+      </c>
+      <c r="F40" s="55" t="inlineStr">
+        <is>
+          <t>Cement 60B + 6mm 50pcs + Gitti + DrFixit + Labour</t>
+        </is>
+      </c>
+      <c r="G40" s="63" t="n">
+        <v>41650</v>
+      </c>
+      <c r="H40" s="55" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I40" s="55" t="n"/>
       <c r="J40" s="55" t="n"/>
-      <c r="K40" s="55" t="n"/>
-      <c r="L40" s="58" t="n"/>
+      <c r="K40" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L40" s="58">
+        <f>L39+G40</f>
+        <v/>
+      </c>
       <c r="M40" s="55" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="99">

</xml_diff>

<commit_message>
Update: Econ Builder ₹15,000 + Iron wire ₹1,300 (Papa, 17-Jul) — iron wiring works
All Transactions rows 525-527:
  - Econ Builder ₹15,000 (engineer supervision — iron wiring)
  - Iron wire 2 Kg @ ₹600 = ₹1,200
  - Iron wire delivery ₹100
Payment Tracker rows 41-42: Papa GPay ₹15,000 + ₹1,300
Excel: 0 errors, 2807 formulas verified.

totalBilled=vendors=categories=monthly=₹15,62,747 ✓
totalPaid=payers=₹17,56,847 ✓  Day 72

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6451,7 +6451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q525"/>
+  <dimension ref="A1:Q528"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -21675,33 +21675,231 @@
       </c>
     </row>
     <row r="525">
-      <c r="A525" s="60" t="inlineStr">
+      <c r="A525" t="n">
+        <v>522</v>
+      </c>
+      <c r="B525" s="127" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C525">
+        <f>IF(B525="","",TEXT(B525,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>Engineer Supervision</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>Engineer supervision fee — iron wiring works</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I525" t="n">
+        <v>1</v>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K525" t="n">
+        <v>15000</v>
+      </c>
+      <c r="L525">
+        <f>IF(OR(I525="",K525=""),"",I525*K525)</f>
+        <v/>
+      </c>
+      <c r="O525">
+        <f>IF(L525="","",IF(M525="",L525,L525*(1-M525)))</f>
+        <v/>
+      </c>
+      <c r="P525" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="Q525" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="n">
+        <v>523</v>
+      </c>
+      <c r="B526" s="127" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C526">
+        <f>IF(B526="","",TEXT(B526,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>Wire</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>Iron wire 2 Kg @ ₹600/kg</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>Local Purchase</t>
+        </is>
+      </c>
+      <c r="I526" t="n">
+        <v>2</v>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>Kg</t>
+        </is>
+      </c>
+      <c r="K526" t="n">
+        <v>600</v>
+      </c>
+      <c r="L526">
+        <f>IF(OR(I526="",K526=""),"",I526*K526)</f>
+        <v/>
+      </c>
+      <c r="O526">
+        <f>IF(L526="","",IF(M526="",L526,L526*(1-M526)))</f>
+        <v/>
+      </c>
+      <c r="P526" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="Q526" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="n">
+        <v>524</v>
+      </c>
+      <c r="B527" s="127" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C527">
+        <f>IF(B527="","",TEXT(B527,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>Iron wire delivery charges</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>Local Purchase</t>
+        </is>
+      </c>
+      <c r="I527" t="n">
+        <v>1</v>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K527" t="n">
+        <v>100</v>
+      </c>
+      <c r="L527">
+        <f>IF(OR(I527="",K527=""),"",I527*K527)</f>
+        <v/>
+      </c>
+      <c r="O527">
+        <f>IF(L527="","",IF(M527="",L527,L527*(1-M527)))</f>
+        <v/>
+      </c>
+      <c r="P527" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="Q527" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B525" s="60" t="n"/>
-      <c r="C525" s="60" t="n"/>
-      <c r="D525" s="60" t="n"/>
-      <c r="E525" s="60" t="n"/>
-      <c r="F525" s="60" t="n"/>
-      <c r="G525" s="60" t="n"/>
-      <c r="H525" s="60" t="n"/>
-      <c r="I525" s="60" t="n"/>
-      <c r="J525" s="60" t="n"/>
-      <c r="K525" s="60" t="n"/>
-      <c r="L525" s="61">
-        <f>SUM(L5:L524)</f>
-        <v/>
-      </c>
-      <c r="M525" s="60" t="n"/>
-      <c r="N525" s="60" t="n"/>
-      <c r="O525" s="61">
-        <f>SUM(O5:O524)</f>
-        <v/>
-      </c>
-      <c r="P525" s="60" t="n"/>
-      <c r="Q525" s="60" t="n"/>
+      <c r="B528" s="60" t="n"/>
+      <c r="C528" s="60" t="n"/>
+      <c r="D528" s="60" t="n"/>
+      <c r="E528" s="60" t="n"/>
+      <c r="F528" s="60" t="n"/>
+      <c r="G528" s="60" t="n"/>
+      <c r="H528" s="60" t="n"/>
+      <c r="I528" s="60" t="n"/>
+      <c r="J528" s="60" t="n"/>
+      <c r="K528" s="60" t="n"/>
+      <c r="L528" s="61">
+        <f>SUM(L5:L527)</f>
+        <v/>
+      </c>
+      <c r="M528" s="60" t="n"/>
+      <c r="N528" s="60" t="n"/>
+      <c r="O528" s="61">
+        <f>SUM(O5:O527)</f>
+        <v/>
+      </c>
+      <c r="P528" s="60" t="n"/>
+      <c r="Q528" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -35377,33 +35575,99 @@
       <c r="M40" s="55" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="99">
-      <c r="A41" s="41" t="n"/>
-      <c r="B41" s="45" t="n"/>
-      <c r="C41" s="47" t="n"/>
-      <c r="D41" s="47" t="n"/>
-      <c r="E41" s="47" t="n"/>
-      <c r="F41" s="47" t="n"/>
-      <c r="G41" s="62" t="n"/>
-      <c r="H41" s="47" t="n"/>
+      <c r="A41" s="41" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="45" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C41" s="47" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D41" s="47" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E41" s="47" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F41" s="47" t="inlineStr">
+        <is>
+          <t>Engineer supervision — iron wiring works</t>
+        </is>
+      </c>
+      <c r="G41" s="62" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H41" s="47" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I41" s="47" t="n"/>
       <c r="J41" s="47" t="n"/>
-      <c r="K41" s="47" t="n"/>
-      <c r="L41" s="50" t="n"/>
+      <c r="K41" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L41" s="50">
+        <f>L40+G41</f>
+        <v/>
+      </c>
       <c r="M41" s="47" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="99">
-      <c r="A42" s="43" t="n"/>
-      <c r="B42" s="53" t="n"/>
-      <c r="C42" s="55" t="n"/>
-      <c r="D42" s="55" t="n"/>
-      <c r="E42" s="55" t="n"/>
-      <c r="F42" s="55" t="n"/>
-      <c r="G42" s="63" t="n"/>
-      <c r="H42" s="55" t="n"/>
+      <c r="A42" s="43" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="53" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C42" s="55" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D42" s="55" t="inlineStr">
+        <is>
+          <t>Local Purchase</t>
+        </is>
+      </c>
+      <c r="E42" s="55" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F42" s="55" t="inlineStr">
+        <is>
+          <t>Iron wire 2kg + delivery</t>
+        </is>
+      </c>
+      <c r="G42" s="63" t="n">
+        <v>1300</v>
+      </c>
+      <c r="H42" s="55" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I42" s="55" t="n"/>
       <c r="J42" s="55" t="n"/>
-      <c r="K42" s="55" t="n"/>
-      <c r="L42" s="58" t="n"/>
+      <c r="K42" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L42" s="58">
+        <f>L41+G42</f>
+        <v/>
+      </c>
       <c r="M42" s="55" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="99">

</xml_diff>

<commit_message>
Update: Econ Builder ₹18,000 (Papa, 17-Jul) — Santosh shuttering work
All Transactions row 528: Prof Fees ₹18,000 — shuttering labour
Payment Tracker row 43: Papa GPay ₹18,000
Excel: 0 errors, 2811 formulas verified.

Econ Builder: ₹3,21,000 → ₹3,39,000 (total paid to engineer)
totalBilled=vendors=categories=monthly=₹15,80,747 ✓
totalPaid=payers=₹17,74,847 ✓

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6451,7 +6451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q528"/>
+  <dimension ref="A1:Q529"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -21873,33 +21873,99 @@
       </c>
     </row>
     <row r="528">
-      <c r="A528" s="60" t="inlineStr">
+      <c r="A528" t="n">
+        <v>525</v>
+      </c>
+      <c r="B528" s="127" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C528">
+        <f>IF(B528="","",TEXT(B528,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>Shuttering Labour</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>Payment to Santosh for shuttering work</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I528" t="n">
+        <v>1</v>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K528" t="n">
+        <v>18000</v>
+      </c>
+      <c r="L528">
+        <f>IF(OR(I528="",K528=""),"",I528*K528)</f>
+        <v/>
+      </c>
+      <c r="O528">
+        <f>IF(L528="","",IF(M528="",L528,L528*(1-M528)))</f>
+        <v/>
+      </c>
+      <c r="P528" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="Q528" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B528" s="60" t="n"/>
-      <c r="C528" s="60" t="n"/>
-      <c r="D528" s="60" t="n"/>
-      <c r="E528" s="60" t="n"/>
-      <c r="F528" s="60" t="n"/>
-      <c r="G528" s="60" t="n"/>
-      <c r="H528" s="60" t="n"/>
-      <c r="I528" s="60" t="n"/>
-      <c r="J528" s="60" t="n"/>
-      <c r="K528" s="60" t="n"/>
-      <c r="L528" s="61">
-        <f>SUM(L5:L527)</f>
-        <v/>
-      </c>
-      <c r="M528" s="60" t="n"/>
-      <c r="N528" s="60" t="n"/>
-      <c r="O528" s="61">
-        <f>SUM(O5:O527)</f>
-        <v/>
-      </c>
-      <c r="P528" s="60" t="n"/>
-      <c r="Q528" s="60" t="n"/>
+      <c r="B529" s="60" t="n"/>
+      <c r="C529" s="60" t="n"/>
+      <c r="D529" s="60" t="n"/>
+      <c r="E529" s="60" t="n"/>
+      <c r="F529" s="60" t="n"/>
+      <c r="G529" s="60" t="n"/>
+      <c r="H529" s="60" t="n"/>
+      <c r="I529" s="60" t="n"/>
+      <c r="J529" s="60" t="n"/>
+      <c r="K529" s="60" t="n"/>
+      <c r="L529" s="61">
+        <f>SUM(L5:L528)</f>
+        <v/>
+      </c>
+      <c r="M529" s="60" t="n"/>
+      <c r="N529" s="60" t="n"/>
+      <c r="O529" s="61">
+        <f>SUM(O5:O528)</f>
+        <v/>
+      </c>
+      <c r="P529" s="60" t="n"/>
+      <c r="Q529" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -35671,18 +35737,51 @@
       <c r="M42" s="55" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="99">
-      <c r="A43" s="41" t="n"/>
-      <c r="B43" s="45" t="n"/>
-      <c r="C43" s="47" t="n"/>
-      <c r="D43" s="47" t="n"/>
-      <c r="E43" s="47" t="n"/>
-      <c r="F43" s="47" t="n"/>
-      <c r="G43" s="62" t="n"/>
-      <c r="H43" s="47" t="n"/>
+      <c r="A43" s="41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="45" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C43" s="47" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D43" s="47" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E43" s="47" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F43" s="47" t="inlineStr">
+        <is>
+          <t>Payment to Santosh for shuttering work</t>
+        </is>
+      </c>
+      <c r="G43" s="62" t="n">
+        <v>18000</v>
+      </c>
+      <c r="H43" s="47" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I43" s="47" t="n"/>
       <c r="J43" s="47" t="n"/>
-      <c r="K43" s="47" t="n"/>
-      <c r="L43" s="50" t="n"/>
+      <c r="K43" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L43" s="50">
+        <f>L42+G43</f>
+        <v/>
+      </c>
       <c r="M43" s="47" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="99">

</xml_diff>

<commit_message>
Fix: Correct 23-Jun entry to 22 trailers (was 20) — Mukesh billed 103,550, Land Dev 94,350, balanceDue 10,350
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -20932,7 +20932,7 @@
       </c>
       <c r="G513" t="inlineStr">
         <is>
-          <t>Mitti filling 20 trailers @ ₹600</t>
+          <t>Mitti filling 22 trailers @ ₹600</t>
         </is>
       </c>
       <c r="H513" t="inlineStr">
@@ -20941,7 +20941,7 @@
         </is>
       </c>
       <c r="I513" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J513" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Mukesh Jul entries: JCB 5hrs + Mitti 86 trailers + Sand 30 trailers = ₹62,600; due now ₹72,950
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -28,13 +28,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="\₹#,##0"/>
     <numFmt numFmtId="165" formatCode="\₹#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="168" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* \-??_);_(@_)"/>
     <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="170" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="39">
     <font>
@@ -529,7 +530,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -786,6 +787,7 @@
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6451,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q529"/>
+  <dimension ref="A1:Q537"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -21939,33 +21941,513 @@
       </c>
     </row>
     <row r="529">
-      <c r="A529" s="60" t="inlineStr">
+      <c r="A529" t="n">
+        <v>526</v>
+      </c>
+      <c r="B529" s="128" t="n">
+        <v>46205</v>
+      </c>
+      <c r="C529">
+        <f>IF(B529="","",TEXT(B529,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Land Development</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>Mitti filling 20 trailers @ ₹600</t>
+        </is>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="I529" t="n">
+        <v>20</v>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>Trailer</t>
+        </is>
+      </c>
+      <c r="K529" t="n">
+        <v>600</v>
+      </c>
+      <c r="L529">
+        <f>IF(OR(I529="",K529=""),"",I529*K529)</f>
+        <v/>
+      </c>
+      <c r="N529">
+        <f>M529*L529</f>
+        <v/>
+      </c>
+      <c r="O529">
+        <f>IF(L529="","",IF(M529="",L529,L529*(1-M529)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="n">
+        <v>527</v>
+      </c>
+      <c r="B530" s="128" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C530">
+        <f>IF(B530="","",TEXT(B530,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>Land Development</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>JCB Work</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>JCB work 60 min (1 hr) @ ₹1,000/hr</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="I530" t="n">
+        <v>1</v>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>Hour</t>
+        </is>
+      </c>
+      <c r="K530" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L530">
+        <f>IF(OR(I530="",K530=""),"",I530*K530)</f>
+        <v/>
+      </c>
+      <c r="N530">
+        <f>M530*L530</f>
+        <v/>
+      </c>
+      <c r="O530">
+        <f>IF(L530="","",IF(M530="",L530,L530*(1-M530)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="n">
+        <v>528</v>
+      </c>
+      <c r="B531" s="128" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C531">
+        <f>IF(B531="","",TEXT(B531,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Land Development</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>Mitti filling 24 trailers @ ₹600</t>
+        </is>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="I531" t="n">
+        <v>24</v>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>Trailer</t>
+        </is>
+      </c>
+      <c r="K531" t="n">
+        <v>600</v>
+      </c>
+      <c r="L531">
+        <f>IF(OR(I531="",K531=""),"",I531*K531)</f>
+        <v/>
+      </c>
+      <c r="N531">
+        <f>M531*L531</f>
+        <v/>
+      </c>
+      <c r="O531">
+        <f>IF(L531="","",IF(M531="",L531,L531*(1-M531)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="n">
+        <v>529</v>
+      </c>
+      <c r="B532" s="128" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C532">
+        <f>IF(B532="","",TEXT(B532,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>Land Development</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>JCB Work</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>JCB work 60 min (1 hr) @ ₹1,000/hr</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="I532" t="n">
+        <v>1</v>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>Hour</t>
+        </is>
+      </c>
+      <c r="K532" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L532">
+        <f>IF(OR(I532="",K532=""),"",I532*K532)</f>
+        <v/>
+      </c>
+      <c r="N532">
+        <f>M532*L532</f>
+        <v/>
+      </c>
+      <c r="O532">
+        <f>IF(L532="","",IF(M532="",L532,L532*(1-M532)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="n">
+        <v>530</v>
+      </c>
+      <c r="B533" s="128" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C533">
+        <f>IF(B533="","",TEXT(B533,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>Land Development</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>Mitti filling 42 trailers @ ₹600</t>
+        </is>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="I533" t="n">
+        <v>42</v>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>Trailer</t>
+        </is>
+      </c>
+      <c r="K533" t="n">
+        <v>600</v>
+      </c>
+      <c r="L533">
+        <f>IF(OR(I533="",K533=""),"",I533*K533)</f>
+        <v/>
+      </c>
+      <c r="N533">
+        <f>M533*L533</f>
+        <v/>
+      </c>
+      <c r="O533">
+        <f>IF(L533="","",IF(M533="",L533,L533*(1-M533)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="n">
+        <v>531</v>
+      </c>
+      <c r="B534" s="128" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C534">
+        <f>IF(B534="","",TEXT(B534,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>Land Development</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>JCB Work</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>JCB work 160 min (2h40m) @ ₹1,000/hr</t>
+        </is>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="I534" t="n">
+        <v>2.666666666666667</v>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>Hour</t>
+        </is>
+      </c>
+      <c r="K534" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L534">
+        <f>IF(OR(I534="",K534=""),"",I534*K534)</f>
+        <v/>
+      </c>
+      <c r="N534">
+        <f>M534*L534</f>
+        <v/>
+      </c>
+      <c r="O534">
+        <f>IF(L534="","",IF(M534="",L534,L534*(1-M534)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="n">
+        <v>532</v>
+      </c>
+      <c r="B535" s="128" t="n">
+        <v>46217</v>
+      </c>
+      <c r="C535">
+        <f>IF(B535="","",TEXT(B535,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>Sand Movement</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>Sand movement 30 trailers @ ₹200</t>
+        </is>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="I535" t="n">
+        <v>30</v>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>Trailer</t>
+        </is>
+      </c>
+      <c r="K535" t="n">
+        <v>200</v>
+      </c>
+      <c r="L535">
+        <f>IF(OR(I535="",K535=""),"",I535*K535)</f>
+        <v/>
+      </c>
+      <c r="N535">
+        <f>M535*L535</f>
+        <v/>
+      </c>
+      <c r="O535">
+        <f>IF(L535="","",IF(M535="",L535,L535*(1-M535)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="n">
+        <v>533</v>
+      </c>
+      <c r="B536" s="128" t="n">
+        <v>46219</v>
+      </c>
+      <c r="C536">
+        <f>IF(B536="","",TEXT(B536,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>Land Development</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>JCB Work</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>JCB work 20 min (0.33 hr) @ ₹1,000/hr</t>
+        </is>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="I536" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>Hour</t>
+        </is>
+      </c>
+      <c r="K536" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L536">
+        <f>IF(OR(I536="",K536=""),"",I536*K536)</f>
+        <v/>
+      </c>
+      <c r="N536">
+        <f>M536*L536</f>
+        <v/>
+      </c>
+      <c r="O536">
+        <f>IF(L536="","",IF(M536="",L536,L536*(1-M536)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B529" s="60" t="n"/>
-      <c r="C529" s="60" t="n"/>
-      <c r="D529" s="60" t="n"/>
-      <c r="E529" s="60" t="n"/>
-      <c r="F529" s="60" t="n"/>
-      <c r="G529" s="60" t="n"/>
-      <c r="H529" s="60" t="n"/>
-      <c r="I529" s="60" t="n"/>
-      <c r="J529" s="60" t="n"/>
-      <c r="K529" s="60" t="n"/>
-      <c r="L529" s="61">
-        <f>SUM(L5:L528)</f>
-        <v/>
-      </c>
-      <c r="M529" s="60" t="n"/>
-      <c r="N529" s="60" t="n"/>
-      <c r="O529" s="61">
+      <c r="B537" s="60" t="n"/>
+      <c r="C537" s="60" t="n"/>
+      <c r="D537" s="60" t="n"/>
+      <c r="E537" s="60" t="n"/>
+      <c r="F537" s="60" t="n"/>
+      <c r="G537" s="60" t="n"/>
+      <c r="H537" s="60" t="n"/>
+      <c r="I537" s="60" t="n"/>
+      <c r="J537" s="60" t="n"/>
+      <c r="K537" s="60" t="n"/>
+      <c r="L537" s="61">
+        <f>SUM(L5:L536)</f>
+        <v/>
+      </c>
+      <c r="M537" s="60" t="n"/>
+      <c r="N537" s="60" t="n"/>
+      <c r="O537" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P529" s="60" t="n"/>
-      <c r="Q529" s="60" t="n"/>
+      <c r="P537" s="60" t="n"/>
+      <c r="Q537" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>

</xml_diff>

<commit_message>
Payment: ₹40,000 to Mukesh Yadav (Self, 18-Jul) — due reduced to ₹32,950
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -36267,17 +36267,47 @@
       <c r="M43" s="47" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="99">
-      <c r="A44" s="43" t="n"/>
-      <c r="B44" s="53" t="n"/>
-      <c r="C44" s="55" t="n"/>
-      <c r="D44" s="55" t="n"/>
-      <c r="E44" s="55" t="n"/>
-      <c r="F44" s="55" t="n"/>
-      <c r="G44" s="63" t="n"/>
-      <c r="H44" s="55" t="n"/>
+      <c r="A44" s="43" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="53" t="n">
+        <v>46221</v>
+      </c>
+      <c r="C44" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D44" s="55" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="E44" s="55" t="inlineStr">
+        <is>
+          <t>Land Development + Labour</t>
+        </is>
+      </c>
+      <c r="F44" s="55" t="inlineStr">
+        <is>
+          <t>JCB + Mitti + Sand movement balance payment</t>
+        </is>
+      </c>
+      <c r="G44" s="63" t="n">
+        <v>40000</v>
+      </c>
+      <c r="H44" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I44" s="55" t="n"/>
       <c r="J44" s="55" t="n"/>
-      <c r="K44" s="55" t="n"/>
+      <c r="K44" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L44" s="58" t="n"/>
       <c r="M44" s="55" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add build_dashboard.py generator: Excel is now single source of truth; standardize Mukesh sub-categories; fix 12-May JCB qty 18->17.5
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -7454,7 +7454,7 @@
       </c>
       <c r="F17" s="47" t="inlineStr">
         <is>
-          <t>Land Levelling/Filling</t>
+          <t>JCB Work</t>
         </is>
       </c>
       <c r="G17" s="47" t="inlineStr">
@@ -7468,7 +7468,7 @@
         </is>
       </c>
       <c r="I17" s="48" t="n">
-        <v>18</v>
+        <v>17.5</v>
       </c>
       <c r="J17" s="47" t="inlineStr">
         <is>
@@ -9229,7 +9229,7 @@
       </c>
       <c r="F43" s="47" t="inlineStr">
         <is>
-          <t>Land Levelling/Filling</t>
+          <t>Mitti Filling</t>
         </is>
       </c>
       <c r="G43" s="47" t="inlineStr">
@@ -9853,7 +9853,7 @@
       </c>
       <c r="F52" s="47" t="inlineStr">
         <is>
-          <t>Land Levelling/Filling</t>
+          <t>Mitti Filling</t>
         </is>
       </c>
       <c r="G52" s="47" t="inlineStr">
@@ -11000,7 +11000,7 @@
       </c>
       <c r="F68" s="47" t="inlineStr">
         <is>
-          <t>Land Levelling/Filling</t>
+          <t>Mitti Filling</t>
         </is>
       </c>
       <c r="G68" s="47" t="inlineStr">
@@ -11144,7 +11144,7 @@
       </c>
       <c r="F70" s="47" t="inlineStr">
         <is>
-          <t>Sand Movement Labour</t>
+          <t>Sand Movement</t>
         </is>
       </c>
       <c r="G70" s="47" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="F71" s="55" t="inlineStr">
         <is>
-          <t>Gitti Movement Labour</t>
+          <t>Gitti Movement</t>
         </is>
       </c>
       <c r="G71" s="55" t="inlineStr">
@@ -20359,7 +20359,7 @@
       </c>
       <c r="F504" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Mitti Filling</t>
         </is>
       </c>
       <c r="G504" t="inlineStr">
@@ -20419,7 +20419,7 @@
       </c>
       <c r="F505" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Mitti Filling</t>
         </is>
       </c>
       <c r="G505" t="inlineStr">
@@ -20749,7 +20749,7 @@
       </c>
       <c r="F510" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Mitti Filling</t>
         </is>
       </c>
       <c r="G510" t="inlineStr">
@@ -20929,7 +20929,7 @@
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Mitti Filling</t>
         </is>
       </c>
       <c r="G513" t="inlineStr">
@@ -21963,7 +21963,7 @@
       </c>
       <c r="F529" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Mitti Filling</t>
         </is>
       </c>
       <c r="G529" t="inlineStr">
@@ -22083,7 +22083,7 @@
       </c>
       <c r="F531" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Mitti Filling</t>
         </is>
       </c>
       <c r="G531" t="inlineStr">
@@ -22203,7 +22203,7 @@
       </c>
       <c r="F533" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Mitti Filling</t>
         </is>
       </c>
       <c r="G533" t="inlineStr">

</xml_diff>

<commit_message>
Payment: ₹5,000 to Econ Builder (Papa, 21-Jul) — advance to Santosh for shuttering work
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q537"/>
+  <dimension ref="A1:Q538"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -22421,33 +22421,93 @@
       </c>
     </row>
     <row r="537">
-      <c r="A537" s="60" t="inlineStr">
+      <c r="A537" t="n">
+        <v>534</v>
+      </c>
+      <c r="B537" s="128" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C537">
+        <f>IF(B537="","",TEXT(B537,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>Shuttering Labour</t>
+        </is>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>Advance to Santosh for shuttering work</t>
+        </is>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I537" t="n">
+        <v>1</v>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>Advance</t>
+        </is>
+      </c>
+      <c r="K537" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L537">
+        <f>IF(OR(I537="",K537=""),"",I537*K537)</f>
+        <v/>
+      </c>
+      <c r="N537">
+        <f>M537*L537</f>
+        <v/>
+      </c>
+      <c r="O537">
+        <f>IF(L537="","",IF(M537="",L537,L537*(1-M537)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B537" s="60" t="n"/>
-      <c r="C537" s="60" t="n"/>
-      <c r="D537" s="60" t="n"/>
-      <c r="E537" s="60" t="n"/>
-      <c r="F537" s="60" t="n"/>
-      <c r="G537" s="60" t="n"/>
-      <c r="H537" s="60" t="n"/>
-      <c r="I537" s="60" t="n"/>
-      <c r="J537" s="60" t="n"/>
-      <c r="K537" s="60" t="n"/>
-      <c r="L537" s="61">
-        <f>SUM(L5:L536)</f>
-        <v/>
-      </c>
-      <c r="M537" s="60" t="n"/>
-      <c r="N537" s="60" t="n"/>
-      <c r="O537" s="61">
+      <c r="B538" s="60" t="n"/>
+      <c r="C538" s="60" t="n"/>
+      <c r="D538" s="60" t="n"/>
+      <c r="E538" s="60" t="n"/>
+      <c r="F538" s="60" t="n"/>
+      <c r="G538" s="60" t="n"/>
+      <c r="H538" s="60" t="n"/>
+      <c r="I538" s="60" t="n"/>
+      <c r="J538" s="60" t="n"/>
+      <c r="K538" s="60" t="n"/>
+      <c r="L538" s="61">
+        <f>SUM(L5:L537)</f>
+        <v/>
+      </c>
+      <c r="M538" s="60" t="n"/>
+      <c r="N538" s="60" t="n"/>
+      <c r="O538" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P537" s="60" t="n"/>
-      <c r="Q537" s="60" t="n"/>
+      <c r="P538" s="60" t="n"/>
+      <c r="Q538" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -36312,17 +36372,47 @@
       <c r="M44" s="55" t="n"/>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="99">
-      <c r="A45" s="41" t="n"/>
-      <c r="B45" s="45" t="n"/>
-      <c r="C45" s="47" t="n"/>
-      <c r="D45" s="47" t="n"/>
-      <c r="E45" s="47" t="n"/>
-      <c r="F45" s="47" t="n"/>
-      <c r="G45" s="62" t="n"/>
-      <c r="H45" s="47" t="n"/>
+      <c r="A45" s="41" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="45" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C45" s="47" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D45" s="47" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E45" s="47" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F45" s="47" t="inlineStr">
+        <is>
+          <t>Payment to Santosh — labour supervision</t>
+        </is>
+      </c>
+      <c r="G45" s="62" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H45" s="47" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I45" s="47" t="n"/>
       <c r="J45" s="47" t="n"/>
-      <c r="K45" s="47" t="n"/>
+      <c r="K45" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L45" s="50" t="n"/>
       <c r="M45" s="47" t="n"/>
     </row>

</xml_diff>

<commit_message>
Payment: ₹22,240 to Pappu Hardware (Self, 21-Jul) — Cement 60 bags + Wire + Transport + Labour
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q538"/>
+  <dimension ref="A1:Q544"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -22481,33 +22481,393 @@
       </c>
     </row>
     <row r="538">
-      <c r="A538" s="60" t="inlineStr">
+      <c r="A538" t="n">
+        <v>535</v>
+      </c>
+      <c r="B538" s="128" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C538">
+        <f>IF(B538="","",TEXT(B538,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>Ultratech Super Cement 30 bags @ ₹350</t>
+        </is>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I538" t="n">
+        <v>30</v>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K538" t="n">
+        <v>350</v>
+      </c>
+      <c r="L538">
+        <f>IF(OR(I538="",K538=""),"",I538*K538)</f>
+        <v/>
+      </c>
+      <c r="N538">
+        <f>M538*L538</f>
+        <v/>
+      </c>
+      <c r="O538">
+        <f>IF(L538="","",IF(M538="",L538,L538*(1-M538)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="n">
+        <v>536</v>
+      </c>
+      <c r="B539" s="128" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C539">
+        <f>IF(B539="","",TEXT(B539,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>Ultratech Plain Cement 30 bags @ ₹330</t>
+        </is>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I539" t="n">
+        <v>30</v>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K539" t="n">
+        <v>330</v>
+      </c>
+      <c r="L539">
+        <f>IF(OR(I539="",K539=""),"",I539*K539)</f>
+        <v/>
+      </c>
+      <c r="N539">
+        <f>M539*L539</f>
+        <v/>
+      </c>
+      <c r="O539">
+        <f>IF(L539="","",IF(M539="",L539,L539*(1-M539)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="n">
+        <v>537</v>
+      </c>
+      <c r="B540" s="128" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C540">
+        <f>IF(B540="","",TEXT(B540,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>Cement freight/transport (Bhada)</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I540" t="n">
+        <v>1</v>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>Trip</t>
+        </is>
+      </c>
+      <c r="K540" t="n">
+        <v>300</v>
+      </c>
+      <c r="L540">
+        <f>IF(OR(I540="",K540=""),"",I540*K540)</f>
+        <v/>
+      </c>
+      <c r="N540">
+        <f>M540*L540</f>
+        <v/>
+      </c>
+      <c r="O540">
+        <f>IF(L540="","",IF(M540="",L540,L540*(1-M540)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="n">
+        <v>538</v>
+      </c>
+      <c r="B541" s="128" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C541">
+        <f>IF(B541="","",TEXT(B541,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>Labour for cement loading/unloading</t>
+        </is>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I541" t="n">
+        <v>1</v>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K541" t="n">
+        <v>240</v>
+      </c>
+      <c r="L541">
+        <f>IF(OR(I541="",K541=""),"",I541*K541)</f>
+        <v/>
+      </c>
+      <c r="N541">
+        <f>M541*L541</f>
+        <v/>
+      </c>
+      <c r="O541">
+        <f>IF(L541="","",IF(M541="",L541,L541*(1-M541)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="n">
+        <v>539</v>
+      </c>
+      <c r="B542" s="128" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C542">
+        <f>IF(B542="","",TEXT(B542,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>Wire</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>Wire 2 bundles</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I542" t="n">
+        <v>2</v>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>Bundle</t>
+        </is>
+      </c>
+      <c r="K542" t="n">
+        <v>600</v>
+      </c>
+      <c r="L542">
+        <f>IF(OR(I542="",K542=""),"",I542*K542)</f>
+        <v/>
+      </c>
+      <c r="N542">
+        <f>M542*L542</f>
+        <v/>
+      </c>
+      <c r="O542">
+        <f>IF(L542="","",IF(M542="",L542,L542*(1-M542)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="n">
+        <v>540</v>
+      </c>
+      <c r="B543" s="128" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C543">
+        <f>IF(B543="","",TEXT(B543,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>Labour for wire handling</t>
+        </is>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I543" t="n">
+        <v>1</v>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K543" t="n">
+        <v>100</v>
+      </c>
+      <c r="L543">
+        <f>IF(OR(I543="",K543=""),"",I543*K543)</f>
+        <v/>
+      </c>
+      <c r="N543">
+        <f>M543*L543</f>
+        <v/>
+      </c>
+      <c r="O543">
+        <f>IF(L543="","",IF(M543="",L543,L543*(1-M543)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B538" s="60" t="n"/>
-      <c r="C538" s="60" t="n"/>
-      <c r="D538" s="60" t="n"/>
-      <c r="E538" s="60" t="n"/>
-      <c r="F538" s="60" t="n"/>
-      <c r="G538" s="60" t="n"/>
-      <c r="H538" s="60" t="n"/>
-      <c r="I538" s="60" t="n"/>
-      <c r="J538" s="60" t="n"/>
-      <c r="K538" s="60" t="n"/>
-      <c r="L538" s="61">
-        <f>SUM(L5:L537)</f>
-        <v/>
-      </c>
-      <c r="M538" s="60" t="n"/>
-      <c r="N538" s="60" t="n"/>
-      <c r="O538" s="61">
+      <c r="B544" s="60" t="n"/>
+      <c r="C544" s="60" t="n"/>
+      <c r="D544" s="60" t="n"/>
+      <c r="E544" s="60" t="n"/>
+      <c r="F544" s="60" t="n"/>
+      <c r="G544" s="60" t="n"/>
+      <c r="H544" s="60" t="n"/>
+      <c r="I544" s="60" t="n"/>
+      <c r="J544" s="60" t="n"/>
+      <c r="K544" s="60" t="n"/>
+      <c r="L544" s="61">
+        <f>SUM(L5:L543)</f>
+        <v/>
+      </c>
+      <c r="M544" s="60" t="n"/>
+      <c r="N544" s="60" t="n"/>
+      <c r="O544" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P538" s="60" t="n"/>
-      <c r="Q538" s="60" t="n"/>
+      <c r="P544" s="60" t="n"/>
+      <c r="Q544" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -36417,17 +36777,47 @@
       <c r="M45" s="47" t="n"/>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="99">
-      <c r="A46" s="43" t="n"/>
-      <c r="B46" s="53" t="n"/>
-      <c r="C46" s="55" t="n"/>
-      <c r="D46" s="55" t="n"/>
-      <c r="E46" s="55" t="n"/>
-      <c r="F46" s="55" t="n"/>
-      <c r="G46" s="63" t="n"/>
-      <c r="H46" s="55" t="n"/>
+      <c r="A46" s="43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="53" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C46" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D46" s="55" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E46" s="55" t="inlineStr">
+        <is>
+          <t>Building Materials + Transport + Labour</t>
+        </is>
+      </c>
+      <c r="F46" s="55" t="inlineStr">
+        <is>
+          <t>Cement 60 bags + wire 2 bundles + transport + labour</t>
+        </is>
+      </c>
+      <c r="G46" s="63" t="n">
+        <v>22240</v>
+      </c>
+      <c r="H46" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I46" s="55" t="n"/>
       <c r="J46" s="55" t="n"/>
-      <c r="K46" s="55" t="n"/>
+      <c r="K46" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L46" s="58" t="n"/>
       <c r="M46" s="55" t="n"/>
     </row>

</xml_diff>

<commit_message>
Fix: Consolidate Babloo Hardware → Pappu Hardware (same vendor); total Pappu ₹533,520
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -21313,7 +21313,7 @@
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>Babloo Hardware</t>
+          <t>Pappu Hardware</t>
         </is>
       </c>
       <c r="I519" t="n">
@@ -21379,7 +21379,7 @@
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>Babloo Hardware</t>
+          <t>Pappu Hardware</t>
         </is>
       </c>
       <c r="I520" t="n">
@@ -21445,7 +21445,7 @@
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>Babloo Hardware</t>
+          <t>Pappu Hardware</t>
         </is>
       </c>
       <c r="I521" t="n">
@@ -21511,7 +21511,7 @@
       </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>Babloo Hardware</t>
+          <t>Pappu Hardware</t>
         </is>
       </c>
       <c r="I522" t="n">
@@ -21577,7 +21577,7 @@
       </c>
       <c r="H523" t="inlineStr">
         <is>
-          <t>Babloo Hardware</t>
+          <t>Pappu Hardware</t>
         </is>
       </c>
       <c r="I523" t="n">
@@ -21643,7 +21643,7 @@
       </c>
       <c r="H524" t="inlineStr">
         <is>
-          <t>Babloo Hardware</t>
+          <t>Pappu Hardware</t>
         </is>
       </c>
       <c r="I524" t="n">
@@ -22528,7 +22528,7 @@
         <v>350</v>
       </c>
       <c r="L538">
-        <f>IF(OR(I538="",K538=""),"",I538*K538)</f>
+        <f>I538*K538</f>
         <v/>
       </c>
       <c r="N538">
@@ -22588,7 +22588,7 @@
         <v>330</v>
       </c>
       <c r="L539">
-        <f>IF(OR(I539="",K539=""),"",I539*K539)</f>
+        <f>I539*K539</f>
         <v/>
       </c>
       <c r="N539">
@@ -22648,7 +22648,7 @@
         <v>300</v>
       </c>
       <c r="L540">
-        <f>IF(OR(I540="",K540=""),"",I540*K540)</f>
+        <f>I540*K540</f>
         <v/>
       </c>
       <c r="N540">
@@ -22708,7 +22708,7 @@
         <v>240</v>
       </c>
       <c r="L541">
-        <f>IF(OR(I541="",K541=""),"",I541*K541)</f>
+        <f>I541*K541</f>
         <v/>
       </c>
       <c r="N541">
@@ -22768,7 +22768,7 @@
         <v>600</v>
       </c>
       <c r="L542">
-        <f>IF(OR(I542="",K542=""),"",I542*K542)</f>
+        <f>I542*K542</f>
         <v/>
       </c>
       <c r="N542">
@@ -22828,7 +22828,7 @@
         <v>100</v>
       </c>
       <c r="L543">
-        <f>IF(OR(I543="",K543=""),"",I543*K543)</f>
+        <f>I543*K543</f>
         <v/>
       </c>
       <c r="N543">
@@ -36508,7 +36508,7 @@
       </c>
       <c r="D40" s="55" t="inlineStr">
         <is>
-          <t>Babloo Hardware</t>
+          <t>Pappu Hardware</t>
         </is>
       </c>
       <c r="E40" s="55" t="inlineStr">

</xml_diff>

<commit_message>
Add 3 Papa payments: 05-Jul ₹25K mitti, 20-Jul ₹22.875K mitti, 20-Jul ₹55.768K food
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q544"/>
+  <dimension ref="A1:Q547"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -22841,33 +22841,213 @@
       </c>
     </row>
     <row r="544">
-      <c r="A544" s="60" t="inlineStr">
+      <c r="A544" t="n">
+        <v>541</v>
+      </c>
+      <c r="B544" s="128" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C544">
+        <f>IF(B544="","",TEXT(B544,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>Daily Labour-Mitti Bharai</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>Mitti bharai additional labour</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>Daily Labour</t>
+        </is>
+      </c>
+      <c r="I544" t="n">
+        <v>1</v>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K544" t="n">
+        <v>25000</v>
+      </c>
+      <c r="L544">
+        <f>I544*K544</f>
+        <v/>
+      </c>
+      <c r="N544">
+        <f>M544*L544</f>
+        <v/>
+      </c>
+      <c r="O544">
+        <f>IF(L544="","",IF(M544="",L544,L544*(1-M544)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="n">
+        <v>542</v>
+      </c>
+      <c r="B545" s="128" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C545">
+        <f>IF(B545="","",TEXT(B545,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>Daily Labour-Mitti Bharai</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>Mitti bharai additional labour</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>Daily Labour</t>
+        </is>
+      </c>
+      <c r="I545" t="n">
+        <v>1</v>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K545" t="n">
+        <v>22875</v>
+      </c>
+      <c r="L545">
+        <f>I545*K545</f>
+        <v/>
+      </c>
+      <c r="N545">
+        <f>M545*L545</f>
+        <v/>
+      </c>
+      <c r="O545">
+        <f>IF(L545="","",IF(M545="",L545,L545*(1-M545)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="n">
+        <v>543</v>
+      </c>
+      <c r="B546" s="128" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C546">
+        <f>IF(B546="","",TEXT(B546,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>Food/Ration</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>Food and miscellaneous provisions</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>Local Purchase</t>
+        </is>
+      </c>
+      <c r="I546" t="n">
+        <v>1</v>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K546" t="n">
+        <v>55768</v>
+      </c>
+      <c r="L546">
+        <f>I546*K546</f>
+        <v/>
+      </c>
+      <c r="N546">
+        <f>M546*L546</f>
+        <v/>
+      </c>
+      <c r="O546">
+        <f>IF(L546="","",IF(M546="",L546,L546*(1-M546)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B544" s="60" t="n"/>
-      <c r="C544" s="60" t="n"/>
-      <c r="D544" s="60" t="n"/>
-      <c r="E544" s="60" t="n"/>
-      <c r="F544" s="60" t="n"/>
-      <c r="G544" s="60" t="n"/>
-      <c r="H544" s="60" t="n"/>
-      <c r="I544" s="60" t="n"/>
-      <c r="J544" s="60" t="n"/>
-      <c r="K544" s="60" t="n"/>
-      <c r="L544" s="61">
-        <f>SUM(L5:L543)</f>
-        <v/>
-      </c>
-      <c r="M544" s="60" t="n"/>
-      <c r="N544" s="60" t="n"/>
-      <c r="O544" s="61">
+      <c r="B547" s="60" t="n"/>
+      <c r="C547" s="60" t="n"/>
+      <c r="D547" s="60" t="n"/>
+      <c r="E547" s="60" t="n"/>
+      <c r="F547" s="60" t="n"/>
+      <c r="G547" s="60" t="n"/>
+      <c r="H547" s="60" t="n"/>
+      <c r="I547" s="60" t="n"/>
+      <c r="J547" s="60" t="n"/>
+      <c r="K547" s="60" t="n"/>
+      <c r="L547" s="61">
+        <f>SUM(L5:L546)</f>
+        <v/>
+      </c>
+      <c r="M547" s="60" t="n"/>
+      <c r="N547" s="60" t="n"/>
+      <c r="O547" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P544" s="60" t="n"/>
-      <c r="Q544" s="60" t="n"/>
+      <c r="P547" s="60" t="n"/>
+      <c r="Q547" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -36781,34 +36961,34 @@
         <v>42</v>
       </c>
       <c r="B46" s="53" t="n">
-        <v>46224</v>
+        <v>46208</v>
       </c>
       <c r="C46" s="55" t="inlineStr">
         <is>
-          <t>Self</t>
+          <t>Papa</t>
         </is>
       </c>
       <c r="D46" s="55" t="inlineStr">
         <is>
-          <t>Pappu Hardware</t>
+          <t>Daily Labour</t>
         </is>
       </c>
       <c r="E46" s="55" t="inlineStr">
         <is>
-          <t>Building Materials + Transport + Labour</t>
+          <t>Labour</t>
         </is>
       </c>
       <c r="F46" s="55" t="inlineStr">
         <is>
-          <t>Cement 60 bags + wire 2 bundles + transport + labour</t>
+          <t>Mitti bharai labour</t>
         </is>
       </c>
       <c r="G46" s="63" t="n">
-        <v>22240</v>
+        <v>25000</v>
       </c>
       <c r="H46" s="55" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>GPay</t>
         </is>
       </c>
       <c r="I46" s="55" t="n"/>
@@ -36822,32 +37002,92 @@
       <c r="M46" s="55" t="n"/>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="99">
-      <c r="A47" s="41" t="n"/>
-      <c r="B47" s="45" t="n"/>
-      <c r="C47" s="47" t="n"/>
-      <c r="D47" s="47" t="n"/>
-      <c r="E47" s="47" t="n"/>
-      <c r="F47" s="47" t="n"/>
-      <c r="G47" s="62" t="n"/>
-      <c r="H47" s="47" t="n"/>
+      <c r="A47" s="41" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="45" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C47" s="47" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D47" s="47" t="inlineStr">
+        <is>
+          <t>Daily Labour</t>
+        </is>
+      </c>
+      <c r="E47" s="47" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F47" s="47" t="inlineStr">
+        <is>
+          <t>Mitti bharai labour</t>
+        </is>
+      </c>
+      <c r="G47" s="62" t="n">
+        <v>22875</v>
+      </c>
+      <c r="H47" s="47" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I47" s="47" t="n"/>
       <c r="J47" s="47" t="n"/>
-      <c r="K47" s="47" t="n"/>
+      <c r="K47" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L47" s="50" t="n"/>
       <c r="M47" s="47" t="n"/>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="99">
-      <c r="A48" s="43" t="n"/>
-      <c r="B48" s="53" t="n"/>
-      <c r="C48" s="55" t="n"/>
-      <c r="D48" s="55" t="n"/>
-      <c r="E48" s="55" t="n"/>
-      <c r="F48" s="55" t="n"/>
-      <c r="G48" s="63" t="n"/>
-      <c r="H48" s="55" t="n"/>
+      <c r="A48" s="43" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="53" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C48" s="55" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D48" s="55" t="inlineStr">
+        <is>
+          <t>Local Purchase</t>
+        </is>
+      </c>
+      <c r="E48" s="55" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F48" s="55" t="inlineStr">
+        <is>
+          <t>Food / Miscellaneous provisions</t>
+        </is>
+      </c>
+      <c r="G48" s="63" t="n">
+        <v>55768</v>
+      </c>
+      <c r="H48" s="55" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I48" s="55" t="n"/>
       <c r="J48" s="55" t="n"/>
-      <c r="K48" s="55" t="n"/>
+      <c r="K48" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L48" s="58" t="n"/>
       <c r="M48" s="55" t="n"/>
     </row>

</xml_diff>

<commit_message>
Fix: Add missing 21-Jul ₹22,240 payment to Pappu Hardware (Self, Cash)
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -37092,17 +37092,47 @@
       <c r="M48" s="55" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="99">
-      <c r="A49" s="41" t="n"/>
-      <c r="B49" s="45" t="n"/>
-      <c r="C49" s="47" t="n"/>
-      <c r="D49" s="47" t="n"/>
-      <c r="E49" s="47" t="n"/>
-      <c r="F49" s="47" t="n"/>
-      <c r="G49" s="62" t="n"/>
-      <c r="H49" s="47" t="n"/>
+      <c r="A49" s="41" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="45" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C49" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D49" s="47" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E49" s="47" t="inlineStr">
+        <is>
+          <t>Building Materials + Transport + Labour</t>
+        </is>
+      </c>
+      <c r="F49" s="47" t="inlineStr">
+        <is>
+          <t>Cement 60 bags + wire + transport + labour</t>
+        </is>
+      </c>
+      <c r="G49" s="62" t="n">
+        <v>22240</v>
+      </c>
+      <c r="H49" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I49" s="47" t="n"/>
       <c r="J49" s="47" t="n"/>
-      <c r="K49" s="47" t="n"/>
+      <c r="K49" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L49" s="50" t="n"/>
       <c r="M49" s="47" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add: 7 tractor brick delivery (22-Jul) — 10,500 bricks @ ₹8.5 = ₹89,250; tractors 14-20
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q547"/>
+  <dimension ref="A1:Q548"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -23021,33 +23021,93 @@
       </c>
     </row>
     <row r="547">
-      <c r="A547" s="60" t="inlineStr">
+      <c r="A547" t="n">
+        <v>541</v>
+      </c>
+      <c r="B547" s="128" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C547">
+        <f>IF(B547="","",TEXT(B547,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>Bricks</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>Brick delivery — tractor 14-20 (10,500 bricks @ ₹8.5)</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>Brick Company</t>
+        </is>
+      </c>
+      <c r="I547" t="n">
+        <v>10500</v>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K547" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="L547">
+        <f>I547*K547</f>
+        <v/>
+      </c>
+      <c r="N547">
+        <f>M547*L547</f>
+        <v/>
+      </c>
+      <c r="O547">
+        <f>IF(L547="","",IF(M547="",L547,L547*(1-M547)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B547" s="60" t="n"/>
-      <c r="C547" s="60" t="n"/>
-      <c r="D547" s="60" t="n"/>
-      <c r="E547" s="60" t="n"/>
-      <c r="F547" s="60" t="n"/>
-      <c r="G547" s="60" t="n"/>
-      <c r="H547" s="60" t="n"/>
-      <c r="I547" s="60" t="n"/>
-      <c r="J547" s="60" t="n"/>
-      <c r="K547" s="60" t="n"/>
-      <c r="L547" s="61">
-        <f>SUM(L5:L546)</f>
-        <v/>
-      </c>
-      <c r="M547" s="60" t="n"/>
-      <c r="N547" s="60" t="n"/>
-      <c r="O547" s="61">
+      <c r="B548" s="60" t="n"/>
+      <c r="C548" s="60" t="n"/>
+      <c r="D548" s="60" t="n"/>
+      <c r="E548" s="60" t="n"/>
+      <c r="F548" s="60" t="n"/>
+      <c r="G548" s="60" t="n"/>
+      <c r="H548" s="60" t="n"/>
+      <c r="I548" s="60" t="n"/>
+      <c r="J548" s="60" t="n"/>
+      <c r="K548" s="60" t="n"/>
+      <c r="L548" s="61">
+        <f>SUM(L5:L547)</f>
+        <v/>
+      </c>
+      <c r="M548" s="60" t="n"/>
+      <c r="N548" s="60" t="n"/>
+      <c r="O548" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P547" s="60" t="n"/>
-      <c r="Q547" s="60" t="n"/>
+      <c r="P548" s="60" t="n"/>
+      <c r="Q548" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>

</xml_diff>